<commit_message>
Add nationalization category/status and import-vs-PAC price comparison
- Tagged 67 low-complexity rows (breakers, connectors, wire/cable,
  harnesses) in Final Cost List with a "Simple Item Category" column
  and a "Nationalization Status" column (already PAC-sourced, high/
  medium/low confidence PAC match, or not comparable).
- Added "Import Scenario" and "Nationalized/PAC Price" columns (BRL,
  including taxes) plus a "Cheaper Option" column, so System/SubSystem
  can be filtered together with nationalization candidates and it's
  visible that nationalizing isn't always cheaper (22 of 64 compared
  items are actually cheaper imported, vs 42 cheaper nationalized).
- Cleared a stray leftover value in column Q.
</commit_message>
<xml_diff>
--- a/Lista_Final_Pathfinder_SKID_Custos_English_Updated.xlsx
+++ b/Lista_Final_Pathfinder_SKID_Custos_English_Updated.xlsx
@@ -122,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -172,6 +172,9 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -957,7 +960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q163"/>
+  <dimension ref="A1:V163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="35.25" customHeight="1"/>
   <cols>
     <col width="42" customWidth="1" style="11" min="1" max="1"/>
@@ -975,8 +978,11 @@
     <col width="29.42578125" customWidth="1" style="11" min="15" max="15"/>
     <col width="97.5703125" bestFit="1" customWidth="1" style="11" min="16" max="16"/>
     <col width="52.85546875" customWidth="1" style="11" min="17" max="18"/>
-    <col width="9.140625" customWidth="1" style="11" min="19" max="19"/>
-    <col width="9.140625" customWidth="1" style="11" min="20" max="16384"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="44" customWidth="1" style="11" min="19" max="19"/>
+    <col width="26" customWidth="1" style="11" min="20" max="16384"/>
+    <col width="26" customWidth="1" min="21" max="21"/>
+    <col width="26" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="35.25" customHeight="1">
@@ -1060,6 +1066,31 @@
           <t>Status / Notes</t>
         </is>
       </c>
+      <c r="R1" s="31" t="inlineStr">
+        <is>
+          <t>Simple Item Category</t>
+        </is>
+      </c>
+      <c r="S1" s="31" t="inlineStr">
+        <is>
+          <t>Nationalization Status</t>
+        </is>
+      </c>
+      <c r="T1" s="31" t="inlineStr">
+        <is>
+          <t>Import Scenario (BOM+TP+Freight+Duty, BRL Incl. Tax)</t>
+        </is>
+      </c>
+      <c r="U1" s="31" t="inlineStr">
+        <is>
+          <t>Nationalized/PAC Price (BRL Incl. Tax)</t>
+        </is>
+      </c>
+      <c r="V1" s="31" t="inlineStr">
+        <is>
+          <t>Cheaper Option</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="35.25" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
@@ -1396,10 +1427,7 @@
           <t>Direct supplier purchase; TP excluded; international freight 9%</t>
         </is>
       </c>
-      <c r="Q7" s="11">
-        <f>63</f>
-        <v/>
-      </c>
+      <c r="Q7" s="11" t="n"/>
     </row>
     <row r="8" ht="35.25" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
@@ -1512,6 +1540,27 @@
           <t>Made by GET; retained for GET impact analysis</t>
         </is>
       </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Wire/Cable</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Low confidence - no comparable PAC item found</t>
+        </is>
+      </c>
+      <c r="T9" s="4" t="n">
+        <v>98621.07208414728</v>
+      </c>
+      <c r="U9" s="4" t="n">
+        <v>7609.408031064615</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 91,011.66)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="35.25" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
@@ -2430,6 +2479,27 @@
           <t>TP included; international freight updated to 9%</t>
         </is>
       </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Wire/Cable</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Low confidence - PAC family match, different length</t>
+        </is>
+      </c>
+      <c r="T26" s="4" t="n">
+        <v>10225.92034333315</v>
+      </c>
+      <c r="U26" s="4" t="n">
+        <v>8409.474282292764</v>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 1,816.45)</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="35.25" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
@@ -2593,6 +2663,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Wire/Cable</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Low confidence - no comparable PAC item found</t>
+        </is>
+      </c>
+      <c r="T29" s="4" t="n">
+        <v>6403.637871675433</v>
+      </c>
+      <c r="U29" s="4" t="n">
+        <v>3569.042073628852</v>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 2,834.60)</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="35.25" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
@@ -2811,6 +2902,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=1.0</t>
         </is>
       </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Wire/Cable</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>High confidence PAC match (exact desc, PN 29707P) - not yet applied</t>
+        </is>
+      </c>
+      <c r="T33" s="4" t="n">
+        <v>4055.495726244304</v>
+      </c>
+      <c r="U33" s="4" t="n">
+        <v>373.698202623823</v>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 3,681.80)</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="35.25" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
@@ -2920,6 +3032,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=1.0</t>
         </is>
       </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T35" s="4" t="n">
+        <v>4406.426976727093</v>
+      </c>
+      <c r="U35" s="4" t="n">
+        <v>3708.649312120554</v>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 697.78)</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="35.25" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
@@ -3133,6 +3266,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Wire/Cable</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T39" s="4" t="n">
+        <v>2660.402040541957</v>
+      </c>
+      <c r="U39" s="4" t="n">
+        <v>2669.977858802905</v>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 9.58)</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="35.25" customHeight="1">
       <c r="A40" s="11" t="inlineStr">
@@ -3398,6 +3552,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Wire/Cable</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Low confidence - PAC match, different length</t>
+        </is>
+      </c>
+      <c r="T44" s="4" t="n">
+        <v>1654.391103723516</v>
+      </c>
+      <c r="U44" s="4" t="n">
+        <v>806.5937814985939</v>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 847.80)</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="35.25" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
@@ -3451,6 +3626,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T45" s="4" t="n">
+        <v>1529.528013903132</v>
+      </c>
+      <c r="U45" s="4" t="n">
+        <v>1626.840122579282</v>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 97.31)</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="35.25" customHeight="1">
       <c r="A46" s="11" t="inlineStr">
@@ -3822,6 +4018,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=1.0</t>
         </is>
       </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T52" s="4" t="n">
+        <v>1028.805161874616</v>
+      </c>
+      <c r="U52" s="4" t="n">
+        <v>1140.991794693213</v>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 112.19)</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="35.25" customHeight="1">
       <c r="A53" s="11" t="inlineStr">
@@ -3873,6 +4090,27 @@
       <c r="P53" s="11" t="inlineStr">
         <is>
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Wire/Cable</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T53" s="4" t="n">
+        <v>975.0172291599222</v>
+      </c>
+      <c r="U53" s="4" t="n">
+        <v>1124.773851951379</v>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 149.76)</t>
         </is>
       </c>
     </row>
@@ -4036,6 +4274,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=1.0</t>
         </is>
       </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Medium confidence PAC match (same PN family - AMP115 backshell)</t>
+        </is>
+      </c>
+      <c r="T56" s="4" t="n">
+        <v>933.6259652062054</v>
+      </c>
+      <c r="U56" s="4" t="n">
+        <v>1034.771349962435</v>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 101.15)</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="35.25" customHeight="1">
       <c r="A57" s="11" t="inlineStr">
@@ -4196,6 +4455,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T59" s="4" t="n">
+        <v>814.0834188901272</v>
+      </c>
+      <c r="U59" s="4" t="n">
+        <v>868.9518208828897</v>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 54.87)</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="35.25" customHeight="1">
       <c r="A60" s="11" t="inlineStr">
@@ -4249,6 +4529,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T60" s="4" t="n">
+        <v>1332.538339679373</v>
+      </c>
+      <c r="U60" s="4" t="n">
+        <v>856.5794292962246</v>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 475.96)</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="35.25" customHeight="1">
       <c r="A61" s="11" t="inlineStr">
@@ -4355,6 +4656,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Low confidence - no comparable PAC item found</t>
+        </is>
+      </c>
+      <c r="T62" s="4" t="n">
+        <v>830.6291937751467</v>
+      </c>
+      <c r="U62" s="4" t="n">
+        <v>836.6164347804548</v>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 5.99)</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="35.25" customHeight="1">
       <c r="A63" s="11" t="inlineStr">
@@ -4408,6 +4730,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T63" s="4" t="n">
+        <v>702.0133912058648</v>
+      </c>
+      <c r="U63" s="4" t="n">
+        <v>783.5079060473141</v>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 81.49)</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="35.25" customHeight="1">
       <c r="A64" s="11" t="inlineStr">
@@ -4461,6 +4804,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>Medium confidence PAC match (same PN family - AMP115 backshell)</t>
+        </is>
+      </c>
+      <c r="T64" s="4" t="n">
+        <v>755.3949779601576</v>
+      </c>
+      <c r="U64" s="4" t="n">
+        <v>1034.771349962435</v>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 279.38)</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="35.25" customHeight="1">
       <c r="A65" s="11" t="inlineStr">
@@ -4514,6 +4878,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=1.0</t>
         </is>
       </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>Low confidence - no current price, weak PAC reference only</t>
+        </is>
+      </c>
+      <c r="T65" s="4" t="n">
+        <v>753.4242756013825</v>
+      </c>
+      <c r="U65" s="4" t="n">
+        <v>166.3661407463061</v>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 587.06)</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="35.25" customHeight="1">
       <c r="A66" s="11" t="inlineStr">
@@ -4567,6 +4952,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Wire/Cable</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Low confidence - PAC candidate is more expensive</t>
+        </is>
+      </c>
+      <c r="T66" s="4" t="n">
+        <v>748.5339371186776</v>
+      </c>
+      <c r="U66" s="4" t="n">
+        <v>1134.271099423992</v>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 385.74)</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="35.25" customHeight="1">
       <c r="A67" s="11" t="inlineStr">
@@ -4620,6 +5026,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Wire/Cable</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>Low confidence - PAC candidate is more expensive</t>
+        </is>
+      </c>
+      <c r="T67" s="4" t="n">
+        <v>748.5339371186776</v>
+      </c>
+      <c r="U67" s="4" t="n">
+        <v>1134.271099423992</v>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 385.74)</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="35.25" customHeight="1">
       <c r="A68" s="11" t="inlineStr">
@@ -4673,6 +5100,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Medium confidence PAC match (same PN family - AMP84 plug)</t>
+        </is>
+      </c>
+      <c r="T68" s="4" t="n">
+        <v>747.5943678314686</v>
+      </c>
+      <c r="U68" s="4" t="n">
+        <v>427.8338351098799</v>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 319.76)</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="35.25" customHeight="1">
       <c r="A69" s="11" t="inlineStr">
@@ -4885,6 +5333,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>Low confidence - family match, wrong sub-type</t>
+        </is>
+      </c>
+      <c r="T72" s="4" t="n">
+        <v>662.3744970338164</v>
+      </c>
+      <c r="U72" s="4" t="n">
+        <v>1034.771349962435</v>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 372.40)</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="35.25" customHeight="1">
       <c r="A73" s="11" t="inlineStr">
@@ -4991,6 +5460,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=3.0</t>
         </is>
       </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>Medium confidence PAC match (same PN family - AMP84 plug)</t>
+        </is>
+      </c>
+      <c r="T74" s="4" t="n">
+        <v>613.9976039668221</v>
+      </c>
+      <c r="U74" s="4" t="n">
+        <v>427.8338351098799</v>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 186.16)</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="35.25" customHeight="1">
       <c r="A75" s="11" t="inlineStr">
@@ -5044,6 +5534,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=3.0</t>
         </is>
       </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>Medium confidence PAC match (same PN family - AMP115 backshell)</t>
+        </is>
+      </c>
+      <c r="T75" s="4" t="n">
+        <v>610.4828032445718</v>
+      </c>
+      <c r="U75" s="4" t="n">
+        <v>1034.771349962435</v>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 424.29)</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="35.25" customHeight="1">
       <c r="A76" s="11" t="inlineStr">
@@ -5098,6 +5609,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=3.0</t>
         </is>
       </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T76" s="4" t="n">
+        <v>927.4217135613918</v>
+      </c>
+      <c r="U76" s="4" t="n">
+        <v>601.5873836463812</v>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 325.83)</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="35.25" customHeight="1">
       <c r="A77" s="11" t="inlineStr">
@@ -5151,6 +5683,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>Low confidence - family match, wrong sub-type</t>
+        </is>
+      </c>
+      <c r="T77" s="4" t="n">
+        <v>598.4837855036034</v>
+      </c>
+      <c r="U77" s="4" t="n">
+        <v>1034.771349962435</v>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 436.29)</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="35.25" customHeight="1">
       <c r="A78" s="11" t="inlineStr">
@@ -5204,6 +5757,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=1.0</t>
         </is>
       </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T78" s="4" t="n">
+        <v>613.8875736129124</v>
+      </c>
+      <c r="U78" s="4" t="n">
+        <v>592.1775922203701</v>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 21.71)</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="35.25" customHeight="1">
       <c r="A79" s="11" t="inlineStr">
@@ -5257,6 +5831,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=3.0</t>
         </is>
       </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>Medium confidence PAC match (same PN family - AMP84 plug)</t>
+        </is>
+      </c>
+      <c r="T79" s="4" t="n">
+        <v>591.0764834486299</v>
+      </c>
+      <c r="U79" s="4" t="n">
+        <v>427.8338351098799</v>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 163.24)</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="35.25" customHeight="1">
       <c r="A80" s="11" t="inlineStr">
@@ -5311,6 +5906,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=3.0</t>
         </is>
       </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T80" s="4" t="n">
+        <v>598.3024855914547</v>
+      </c>
+      <c r="U80" s="4" t="n">
+        <v>570.9985723265715</v>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 27.30)</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="35.25" customHeight="1">
       <c r="A81" s="11" t="inlineStr">
@@ -5364,6 +5980,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=3.0</t>
         </is>
       </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T81" s="4" t="n">
+        <v>603.5609611549813</v>
+      </c>
+      <c r="U81" s="4" t="n">
+        <v>568.1316302975433</v>
+      </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 35.43)</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="35.25" customHeight="1">
       <c r="A82" s="11" t="inlineStr">
@@ -5417,6 +6054,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=3.0</t>
         </is>
       </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T82" s="4" t="n">
+        <v>552.4752458153932</v>
+      </c>
+      <c r="U82" s="4" t="n">
+        <v>555.5830253154769</v>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 3.11)</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="35.25" customHeight="1">
       <c r="A83" s="11" t="inlineStr">
@@ -5471,6 +6129,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=3.0</t>
         </is>
       </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T83" s="4" t="n">
+        <v>643.0350314673822</v>
+      </c>
+      <c r="U83" s="4" t="n">
+        <v>534.8246954151087</v>
+      </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 108.21)</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="35.25" customHeight="1">
       <c r="A84" s="11" t="inlineStr">
@@ -5524,6 +6203,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T84" s="4" t="n">
+        <v>582.4018101393276</v>
+      </c>
+      <c r="U84" s="4" t="n">
+        <v>515.8462233909341</v>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 66.56)</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="35.25" customHeight="1">
       <c r="A85" s="11" t="inlineStr">
@@ -5631,6 +6331,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T86" s="4" t="n">
+        <v>534.2875477016347</v>
+      </c>
+      <c r="U86" s="4" t="n">
+        <v>484.0301325820185</v>
+      </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 50.26)</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="35.25" customHeight="1">
       <c r="A87" s="11" t="inlineStr">
@@ -5684,6 +6405,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>Medium confidence PAC match (same PN family - AMP84 plug)</t>
+        </is>
+      </c>
+      <c r="T87" s="4" t="n">
+        <v>482.4266888310744</v>
+      </c>
+      <c r="U87" s="4" t="n">
+        <v>427.8338351098799</v>
+      </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 54.59)</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="35.25" customHeight="1">
       <c r="A88" s="11" t="inlineStr">
@@ -5738,6 +6480,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>Low confidence - generic family match only</t>
+        </is>
+      </c>
+      <c r="T88" s="4" t="n">
+        <v>475.8777972544481</v>
+      </c>
+      <c r="U88" s="4" t="n">
+        <v>333.0638522909267</v>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 142.81)</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="35.25" customHeight="1">
       <c r="A89" s="11" t="inlineStr">
@@ -5897,6 +6660,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T91" s="4" t="n">
+        <v>621.263443594086</v>
+      </c>
+      <c r="U91" s="4" t="n">
+        <v>419.6026292225457</v>
+      </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 201.66)</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="35.25" customHeight="1">
       <c r="A92" s="11" t="inlineStr">
@@ -5950,6 +6734,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=3.0</t>
         </is>
       </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T92" s="4" t="n">
+        <v>362.6947719609851</v>
+      </c>
+      <c r="U92" s="4" t="n">
+        <v>383.8685749742605</v>
+      </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 21.17)</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="35.25" customHeight="1">
       <c r="A93" s="11" t="inlineStr">
@@ -6004,6 +6809,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T93" s="4" t="n">
+        <v>360.4846737355794</v>
+      </c>
+      <c r="U93" s="4" t="n">
+        <v>353.6260534632618</v>
+      </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 6.86)</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="35.25" customHeight="1">
       <c r="A94" s="11" t="inlineStr">
@@ -6058,6 +6884,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T94" s="4" t="n">
+        <v>337.8521239029884</v>
+      </c>
+      <c r="U94" s="4" t="n">
+        <v>329.058658197743</v>
+      </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 8.79)</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="35.25" customHeight="1">
       <c r="A95" s="11" t="inlineStr">
@@ -6164,6 +7011,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>High confidence PAC match (exact PN) - not yet applied</t>
+        </is>
+      </c>
+      <c r="T96" s="4" t="n">
+        <v>229.1238033877614</v>
+      </c>
+      <c r="U96" s="4" t="n">
+        <v>94.30396293586904</v>
+      </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 134.82)</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="35.25" customHeight="1">
       <c r="A97" s="11" t="inlineStr">
@@ -6271,6 +7139,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T98" s="4" t="n">
+        <v>189.0930849819815</v>
+      </c>
+      <c r="U98" s="4" t="n">
+        <v>192.6883226396193</v>
+      </c>
+      <c r="V98" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 3.60)</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="35.25" customHeight="1">
       <c r="A99" s="11" t="inlineStr">
@@ -6325,6 +7214,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T99" s="4" t="n">
+        <v>188.9579741132262</v>
+      </c>
+      <c r="U99" s="4" t="n">
+        <v>192.5065232295773</v>
+      </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 3.55)</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="35.25" customHeight="1">
       <c r="A100" s="11" t="inlineStr">
@@ -6378,6 +7288,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T100" s="4" t="n">
+        <v>192.0645378838769</v>
+      </c>
+      <c r="U100" s="4" t="n">
+        <v>190.8173559267836</v>
+      </c>
+      <c r="V100" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 1.25)</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="35.25" customHeight="1">
       <c r="A101" s="11" t="inlineStr">
@@ -6431,6 +7362,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T101" s="4" t="n">
+        <v>224.95466542394</v>
+      </c>
+      <c r="U101" s="4" t="n">
+        <v>189.9890376422986</v>
+      </c>
+      <c r="V101" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 34.97)</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="35.25" customHeight="1">
       <c r="A102" s="11" t="inlineStr">
@@ -6537,6 +7489,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T103" s="4" t="n">
+        <v>217.1695179936174</v>
+      </c>
+      <c r="U103" s="4" t="n">
+        <v>186.2575318741715</v>
+      </c>
+      <c r="V103" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 30.91)</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="35.25" customHeight="1">
       <c r="A104" s="11" t="inlineStr">
@@ -6590,6 +7563,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=25.0</t>
         </is>
       </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T104" s="4" t="n">
+        <v>186.2952051669542</v>
+      </c>
+      <c r="U104" s="4" t="n">
+        <v>179.5701278719118</v>
+      </c>
+      <c r="V104" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 6.73)</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="35.25" customHeight="1">
       <c r="A105" s="11" t="inlineStr">
@@ -6749,6 +7743,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T107" s="4" t="n">
+        <v>189.1552162573945</v>
+      </c>
+      <c r="U107" s="4" t="n">
+        <v>156.8498075721028</v>
+      </c>
+      <c r="V107" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 32.31)</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="35.25" customHeight="1">
       <c r="A108" s="11" t="inlineStr">
@@ -6802,6 +7817,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T108" s="4" t="n">
+        <v>159.7168262402766</v>
+      </c>
+      <c r="U108" s="4" t="n">
+        <v>145.4632556175288</v>
+      </c>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 14.25)</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="35.25" customHeight="1">
       <c r="A109" s="11" t="inlineStr">
@@ -6855,6 +7891,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>Low confidence - PAC price range too wide (R$118-2,748)</t>
+        </is>
+      </c>
+      <c r="T109" s="4" t="n">
+        <v>142.1319652632908</v>
+      </c>
+      <c r="U109" s="4" t="n">
+        <v>574.7190868112949</v>
+      </c>
+      <c r="V109" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 432.59)</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="35.25" customHeight="1">
       <c r="A110" s="11" t="inlineStr">
@@ -6908,6 +7965,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T110" s="4" t="n">
+        <v>122.2546257983923</v>
+      </c>
+      <c r="U110" s="4" t="n">
+        <v>135.3758719381956</v>
+      </c>
+      <c r="V110" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 13.12)</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="35.25" customHeight="1">
       <c r="A111" s="11" t="inlineStr">
@@ -7068,6 +8146,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T113" s="4" t="n">
+        <v>117.404441473294</v>
+      </c>
+      <c r="U113" s="4" t="n">
+        <v>92.21012065565543</v>
+      </c>
+      <c r="V113" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 25.19)</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="35.25" customHeight="1">
       <c r="A114" s="11" t="inlineStr">
@@ -7121,6 +8220,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T114" s="4" t="n">
+        <v>92.90104990326674</v>
+      </c>
+      <c r="U114" s="4" t="n">
+        <v>89.56395955578907</v>
+      </c>
+      <c r="V114" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 3.34)</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="35.25" customHeight="1">
       <c r="A115" s="11" t="inlineStr">
@@ -7227,6 +8347,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S116" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T116" s="4" t="n">
+        <v>89.69389263909028</v>
+      </c>
+      <c r="U116" s="4" t="n">
+        <v>82.20453587528175</v>
+      </c>
+      <c r="V116" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 7.49)</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="35.25" customHeight="1">
       <c r="A117" s="11" t="inlineStr">
@@ -7280,6 +8421,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S117" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T117" s="4" t="n">
+        <v>79.72527467282467</v>
+      </c>
+      <c r="U117" s="4" t="n">
+        <v>77.66739248808081</v>
+      </c>
+      <c r="V117" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 2.06)</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="35.25" customHeight="1">
       <c r="A118" s="11" t="inlineStr">
@@ -7386,6 +8548,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S119" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T119" s="4" t="n">
+        <v>53.94572643002858</v>
+      </c>
+      <c r="U119" s="4" t="n">
+        <v>52.72196887330579</v>
+      </c>
+      <c r="V119" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 1.22)</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="35.25" customHeight="1">
       <c r="A120" s="11" t="inlineStr">
@@ -7492,6 +8675,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S121" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T121" s="4" t="n">
+        <v>48.25430436005243</v>
+      </c>
+      <c r="U121" s="4" t="n">
+        <v>44.45710986726772</v>
+      </c>
+      <c r="V121" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 3.80)</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="35.25" customHeight="1">
       <c r="A122" s="11" t="inlineStr">
@@ -7544,6 +8748,19 @@
         <is>
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>Wire/Cable</t>
+        </is>
+      </c>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="U122" s="4" t="n">
+        <v>39.7487438177525</v>
       </c>
     </row>
     <row r="123" ht="35.25" customHeight="1">
@@ -7601,6 +8818,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T123" s="4" t="n">
+        <v>36.25359920349296</v>
+      </c>
+      <c r="U123" s="4" t="n">
+        <v>30.14404395022202</v>
+      </c>
+      <c r="V123" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 6.11)</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="35.25" customHeight="1">
       <c r="A124" s="11" t="inlineStr">
@@ -7707,6 +8945,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>Low confidence - negligible value, family match only</t>
+        </is>
+      </c>
+      <c r="T125" s="4" t="n">
+        <v>20.07535972027769</v>
+      </c>
+      <c r="U125" s="4" t="n">
+        <v>18.57964198750939</v>
+      </c>
+      <c r="V125" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 1.50)</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="35.25" customHeight="1">
       <c r="A126" s="11" t="inlineStr">
@@ -7760,6 +9019,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T126" s="4" t="n">
+        <v>18.0249733448196</v>
+      </c>
+      <c r="U126" s="4" t="n">
+        <v>17.78537526901411</v>
+      </c>
+      <c r="V126" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 0.24)</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="35.25" customHeight="1">
       <c r="A127" s="11" t="inlineStr">
@@ -7814,6 +9094,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T127" s="4" t="n">
+        <v>16.64526454636238</v>
+      </c>
+      <c r="U127" s="4" t="n">
+        <v>16.43514113685199</v>
+      </c>
+      <c r="V127" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 0.21)</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="35.25" customHeight="1">
       <c r="A128" s="11" t="inlineStr">
@@ -7868,6 +9169,27 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T128" s="4" t="n">
+        <v>16.30995290127628</v>
+      </c>
+      <c r="U128" s="4" t="n">
+        <v>15.8008918171641</v>
+      </c>
+      <c r="V128" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 0.51)</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="35.25" customHeight="1">
       <c r="A129" s="11" t="inlineStr">
@@ -8080,6 +9402,27 @@
           <t>Calculated with TP (17.2%) + International Freight (15%) + Import Duty (16%) + Domestic Freight (3%) | Qtd=1.0</t>
         </is>
       </c>
+      <c r="R132" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T132" s="4" t="n">
+        <v>8.868006801806525</v>
+      </c>
+      <c r="U132" s="4" t="n">
+        <v>9.197715577855137</v>
+      </c>
+      <c r="V132" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 0.33)</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="35.25" customHeight="1">
       <c r="A133" s="11" t="inlineStr">
@@ -8186,6 +9529,27 @@
           <t>Item included in the master kit or with no additional cost</t>
         </is>
       </c>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S134" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T134" s="4" t="n">
+        <v>7.262455748276607</v>
+      </c>
+      <c r="U134" s="4" t="n">
+        <v>6.490932858961039</v>
+      </c>
+      <c r="V134" t="inlineStr">
+        <is>
+          <t>PAC/National is cheaper (by R$ 0.77)</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="35.25" customHeight="1">
       <c r="A135" s="11" t="inlineStr">
@@ -8239,6 +9603,27 @@
           <t>Recovered from Pathfinder BOM (Smart Light Source Co.); had no Part Number so was missed by PN-based matching. TP included (not yet color-reviewed, treated as default Yellow); freight 9%.</t>
         </is>
       </c>
+      <c r="R135" t="inlineStr">
+        <is>
+          <t>Connector/Plug</t>
+        </is>
+      </c>
+      <c r="S135" t="inlineStr">
+        <is>
+          <t>Already nationalized (PAC)</t>
+        </is>
+      </c>
+      <c r="T135" s="4" t="n">
+        <v>1.568075046137942</v>
+      </c>
+      <c r="U135" s="4" t="n">
+        <v>1.723022640070123</v>
+      </c>
+      <c r="V135" t="inlineStr">
+        <is>
+          <t>Import is cheaper (by R$ 0.15)</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="35.25" customHeight="1">
       <c r="A136" s="11" t="inlineStr">
@@ -8345,6 +9730,23 @@
           <t>Quotation pending (no USD or BRL price)</t>
         </is>
       </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>Wire/Cable</t>
+        </is>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>Low confidence - current BOM price is a $0.01 placeholder</t>
+        </is>
+      </c>
+      <c r="T137" s="4" t="n"/>
+      <c r="U137" s="4" t="n"/>
+      <c r="V137" t="inlineStr">
+        <is>
+          <t>Not comparable - current price is a $0.01 BOM placeholder</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="35.25" customHeight="1">
       <c r="A138" s="11" t="inlineStr">
@@ -8396,6 +9798,23 @@
       <c r="P138" s="11" t="inlineStr">
         <is>
           <t>Quotation pending (no USD or BRL price)</t>
+        </is>
+      </c>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>Wire/Cable</t>
+        </is>
+      </c>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>Low confidence - current BOM price is a $0.01 placeholder</t>
+        </is>
+      </c>
+      <c r="T138" s="4" t="n"/>
+      <c r="U138" s="4" t="n"/>
+      <c r="V138" t="inlineStr">
+        <is>
+          <t>Not comparable - current price is a $0.01 BOM placeholder</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Freight Handoff sheet with raw US cost, excluding PAC items
- New "Freight Handoff" sheet lists only the 74 non-PAC items (Imported
  BOM/GET/Missing), since PAC-sourced items already have TP, all
  freight, and import duty baked into their price.
- Shows the raw US unit/total cost (no markup) plus weight, dimensions,
  NCM, and weight confidence, so the freight team can apply Transfer
  Price, international/domestic freight, and import duty themselves.
- AutoFilter enabled on the header row (row 2, row 1 is an explanatory
  note) so every column can be filtered in Excel.
</commit_message>
<xml_diff>
--- a/Lista_Final_Pathfinder_SKID_Custos_English_Updated.xlsx
+++ b/Lista_Final_Pathfinder_SKID_Custos_English_Updated.xlsx
@@ -3,16 +3,18 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary (GDT Project)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final Cost List" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDT Integration and Assembly" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missing Items" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Freight Handoff" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Final Cost List'!$A$1:$O$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Freight Handoff'!$A$2:$M$76</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +27,7 @@
     <numFmt numFmtId="165" formatCode="\$\ #,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,8 +84,21 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FFCC0000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF808080"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -140,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -196,6 +211,8 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -978,7 +995,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AA163"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="26" defaultRowHeight="35.25" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="18" defaultRowHeight="35.25" customHeight="1"/>
   <cols>
     <col width="42" customWidth="1" style="8" min="1" max="1"/>
     <col width="39" customWidth="1" style="8" min="2" max="2"/>
@@ -1000,11 +1017,11 @@
     <col width="44" customWidth="1" style="8" min="19" max="19"/>
     <col width="26" customWidth="1" style="8" min="20" max="20"/>
     <col width="26" customWidth="1" min="21" max="22"/>
-    <col width="18" customWidth="1" style="8" min="23" max="16384"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
-    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" style="8" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="25"/>
     <col width="55" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" style="8" min="28" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="35.25" customHeight="1">
@@ -14421,4 +14438,2869 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M76"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="7"/>
+    <col width="13" customWidth="1" min="8" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="32" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>Part Number</t>
+        </is>
+      </c>
+      <c r="B1" s="30" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="30" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D1" s="30" t="inlineStr">
+        <is>
+          <t>SubSystem</t>
+        </is>
+      </c>
+      <c r="E1" s="30" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="F1" s="30" t="inlineStr">
+        <is>
+          <t>US Unit Cost (USD, no markup)</t>
+        </is>
+      </c>
+      <c r="G1" s="30" t="inlineStr">
+        <is>
+          <t>US Total Cost (USD, no markup)</t>
+        </is>
+      </c>
+      <c r="H1" s="30" t="inlineStr">
+        <is>
+          <t>Unit Weight (kg)</t>
+        </is>
+      </c>
+      <c r="I1" s="30" t="inlineStr">
+        <is>
+          <t>Total Weight (kg)</t>
+        </is>
+      </c>
+      <c r="J1" s="30" t="inlineStr">
+        <is>
+          <t>Dimensions (C x A x L, in)</t>
+        </is>
+      </c>
+      <c r="K1" s="30" t="inlineStr">
+        <is>
+          <t>NCM</t>
+        </is>
+      </c>
+      <c r="L1" s="30" t="inlineStr">
+        <is>
+          <t>Weight Confidence</t>
+        </is>
+      </c>
+      <c r="M1" s="30" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="31" t="inlineStr">
+        <is>
+          <t>41A296352CMP437</t>
+        </is>
+      </c>
+      <c r="B2" s="31" t="inlineStr">
+        <is>
+          <t>Dual Processor Module (DPM)+ LXA (Distributed Power Radio)</t>
+        </is>
+      </c>
+      <c r="C2" s="31" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D2" s="31" t="inlineStr">
+        <is>
+          <t>LXA</t>
+        </is>
+      </c>
+      <c r="E2" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="31" t="n">
+        <v>63100.8192</v>
+      </c>
+      <c r="G2" s="31" t="n">
+        <v>63100.8192</v>
+      </c>
+      <c r="H2" s="31" t="n">
+        <v>4.536</v>
+      </c>
+      <c r="I2" s="31" t="n">
+        <v>4.536</v>
+      </c>
+      <c r="J2" s="31" t="n"/>
+      <c r="K2" s="31" t="inlineStr">
+        <is>
+          <t>90328990</t>
+        </is>
+      </c>
+      <c r="L2" s="31" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M2" s="31" t="inlineStr">
+        <is>
+          <t>FLAGGED - weight looks wrong, verify</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>41A296352LUG24</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CSX Antenna Enclosure Arrangement</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Connectivity</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ANTENNA KIT Master</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G3" t="n">
+        <v>30000</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>37495P</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>KIT ETMS VIRGIN TRAINS FEC EVO44</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PTC KIT MASTER</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>28529</v>
+      </c>
+      <c r="G4" t="n">
+        <v>28529</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>84A215295P62</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Pneumatic Brake Control System (Including lament and control portions) Includes EM EAB Control Functionality</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Fastbrake</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>23409.1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>23409.1</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>41A296352DNP37</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>RADIO PRAD PTC RADIO</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G6" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>84A222059P5</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BATTERIES</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>POWER</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>15685.42</v>
+      </c>
+      <c r="G7" t="n">
+        <v>31370.84</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>84A237085AEP121</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>8 Slot ACC Chassis for MCA w/ i7 HPEAP and SMM2 Cards</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>TRAIN CONTROL</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G8" t="n">
+        <v>8000</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>17KC108E28</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MASTER CONTROLLER</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>TRAIN CONTROL</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5877.102</v>
+      </c>
+      <c r="G9" t="n">
+        <v>5877.102</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>84A215295P73</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Air Brake Handle Assembly (AAR Console)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Fastbrake</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5702.83</v>
+      </c>
+      <c r="G10" t="n">
+        <v>5702.83</v>
+      </c>
+      <c r="H10" t="n">
+        <v>29.03</v>
+      </c>
+      <c r="I10" t="n">
+        <v>29.03</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Weight is an estimate (similar item)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>17FM878A6</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>NIO 2.0</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>MCA</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>5176.9118</v>
+      </c>
+      <c r="G11" t="n">
+        <v>15530.7354</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>L7000083-900</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Wireless Communications Management Module, Gen 3 (WCM3)​</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>TRAIN CONTROL</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G12" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>17FM868B2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SNIO</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MCA</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4150.9559</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4150.9559</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>41A296352DNP55</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>VOICE RADIO RITRON</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Connectivity</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>VOICE RADIO</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>3933</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3933</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>32613P</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>KIT ETMS AXLE INTERFACE FOR WPart Number 29266P</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2981.71</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2981.71</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>41B546155P2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Horn</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>TRAIN CONTROL</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1891.99</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1891.99</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>41D758679BJG16 	84D704379AFG1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>EC Part NumberL ASM</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Circuit Breaker</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1572.36</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1572.36</v>
+      </c>
+      <c r="H17" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="I17" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>20x3.5x25.5</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>86079100</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>84A215295P3</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>POU-to-Handle cable 18' length</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Fastbrake</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1036.89</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1036.89</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1.247</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1.247</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Weight is an estimate (similar item)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Ditchlight Control Box (SMART BOX-V3-DLC )</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>TRAIN CONTROL</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" t="n">
+        <v>800</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1600</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>RCCR-RMTCBL-RA-CUSTOM</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>VOICE RADIO RITRON CABLE,REMOTE,RR-225/XXX, RCCR,RIGHT
+ANGLE,19-PIN,FLAME RETARDANT</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Connectivity</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>VOICE RADIO</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>761</v>
+      </c>
+      <c r="G20" t="n">
+        <v>761</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>41A296352PTP306/41A296352PTP122</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Assembled Air Manifold (Contains 3 pressure sensors mounted in appropriate locations on Air Manifold.)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>595.7889</v>
+      </c>
+      <c r="G21" t="n">
+        <v>595.7889</v>
+      </c>
+      <c r="H21" t="n">
+        <v>5.897</v>
+      </c>
+      <c r="I21" t="n">
+        <v>5.897</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>85381000</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Weight is an estimate (similar item)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>32447P</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ASY CABLE WHEEL TACH AC EVO/SD70 ACE</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>411.22</v>
+      </c>
+      <c r="G22" t="n">
+        <v>411.22</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>41A296352PTP10/319/34</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>VALVE Part NumberEUMATIC NC/CO (Penalty Magnet Valve) Graham-White 812-142</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="n">
+        <v>404.6239</v>
+      </c>
+      <c r="G23" t="n">
+        <v>404.6239</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>LED Ditch Light</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>TRAIN CONTROL</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>4</v>
+      </c>
+      <c r="F24" t="n">
+        <v>375</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>84A231123CSP30</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Axle Tac - WRE Part Number: 29266P</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>205</v>
+      </c>
+      <c r="G25" t="n">
+        <v>205</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>84A201850P4</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ENGINE CONTROL SWITCH</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>TRAIN CONTROL</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>171.544</v>
+      </c>
+      <c r="G26" t="n">
+        <v>171.544</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>RCCR-PWRCBL</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CABLE, PWR, 72V,RA,6.5FT (78").,RR-070,RCCR</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Connectivity</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>VOICE RADIO</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>159</v>
+      </c>
+      <c r="G27" t="n">
+        <v>159</v>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>17 pin MS3106-20-29F</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Head of Train Device - Padom - J2 Connector</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>79.83</v>
+      </c>
+      <c r="G28" t="n">
+        <v>79.83</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>5088-7000-P4611-0000000-ND‎</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>POE Power Connector on SMM2 (M12 FEMALE 0 L-CODED FIELD-WIREA)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>TRAIN CONTROL</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="n">
+        <v>72.41</v>
+      </c>
+      <c r="G29" t="n">
+        <v>72.41</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>41A296352PTP67</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>CABLE CSX 12V P WR CBL</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>MCA</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" t="n">
+        <v>71.94</v>
+      </c>
+      <c r="G30" t="n">
+        <v>71.94</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>41A296352PTP69</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>CABLE CSX 74V P WR CBL</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>MCA</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>71.94</v>
+      </c>
+      <c r="G31" t="n">
+        <v>71.94</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>16246P</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Flexi-Axle - WRE Part Number: 16246P</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="n">
+        <v>59.75</v>
+      </c>
+      <c r="G32" t="n">
+        <v>59.75</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>41A216641ABP153</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>HELPER'S RADIO SPEAKER 
+CONNECTOR</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>45.7356</v>
+      </c>
+      <c r="G33" t="n">
+        <v>45.7356</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>41A216641AMP126</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>NIO1D CONNECTOR BACKSHELL</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>3</v>
+      </c>
+      <c r="F34" t="n">
+        <v>29.9096</v>
+      </c>
+      <c r="G34" t="n">
+        <v>89.72880000000001</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>0x0x0</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>41A216641AMP125</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>NIO1A CONNECTOR BACKSHELL</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>3</v>
+      </c>
+      <c r="F35" t="n">
+        <v>24.1998</v>
+      </c>
+      <c r="G35" t="n">
+        <v>72.5994</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>0x0x0</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>41A216641AMP93</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>NIO1E CONNECTOR</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>3</v>
+      </c>
+      <c r="F36" t="n">
+        <v>23.9499</v>
+      </c>
+      <c r="G36" t="n">
+        <v>71.8497</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.162</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>0x0x0</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>41A212414P31, 41A212414P3 2-Pole Option</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>AUTOCOUPLER CIRCUIT BREAKER,  CCB(2A)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Circuit Breaker</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="n">
+        <v>22.0206</v>
+      </c>
+      <c r="G37" t="n">
+        <v>22.0206</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.093</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.093</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>2.5x0.65x3.05</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>85362000</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>41A216641AMP103</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>NIO1D CONNECTOR</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" t="n">
+        <v>21.2198</v>
+      </c>
+      <c r="G38" t="n">
+        <v>63.6594</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>1.5x1x1.5</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>41A216641AMP99</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>NIO1B CONNECTOR</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>3</v>
+      </c>
+      <c r="F39" t="n">
+        <v>19.67</v>
+      </c>
+      <c r="G39" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>0x0x0</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>41A216641AMP123</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>NIO1F CONNECTOR BACKSHELL</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" t="n">
+        <v>19.5574</v>
+      </c>
+      <c r="G40" t="n">
+        <v>58.6722</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>0x0x0</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>41A216641AMP100</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>NIO1C CONNECTOR</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" t="n">
+        <v>19.173</v>
+      </c>
+      <c r="G41" t="n">
+        <v>57.519</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>0x0x0</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>41A216641AMP86</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>NIO1F CONNECTOR</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" t="n">
+        <v>18.9357</v>
+      </c>
+      <c r="G42" t="n">
+        <v>56.8071</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>3.95x1.25x6.65</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>41A216641AMP98</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>NIO1A CONNECTOR</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" t="n">
+        <v>15.455</v>
+      </c>
+      <c r="G43" t="n">
+        <v>46.365</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.159</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>0x0x0</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>5373-219</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>CONNECTOR, ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="n">
+        <v>13.66</v>
+      </c>
+      <c r="G44" t="n">
+        <v>13.66</v>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>84A207079ABP1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>41A313392DCP18 alternative 300" /</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>25</v>
+      </c>
+      <c r="F45" t="n">
+        <v>8.118</v>
+      </c>
+      <c r="G45" t="n">
+        <v>202.95</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.227</v>
+      </c>
+      <c r="I45" t="n">
+        <v>5.675</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>24x20x24</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>85446000</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>41A271471P24/38</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>HPEAP DISCRETE CONNECTOR Backshell</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1.9294</v>
+      </c>
+      <c r="G46" t="n">
+        <v>1.9294</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>5.1x1.15x2.95</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>85366990</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>41A296352DNP73</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>CABLE: GROUND S TRAP</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>MCA</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>41A296352DNP96</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Cable: CRM Ethernet Switch to ACC</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>MCA</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="32" t="inlineStr">
+        <is>
+          <t>US cost only - no Transfer Price, freight, or import duty applied. PAC-sourced items are excluded (their PAC price already includes TP + all freight + import duty).</t>
+        </is>
+      </c>
+      <c r="B49" s="32" t="n"/>
+      <c r="C49" s="32" t="n"/>
+      <c r="D49" s="32" t="n"/>
+      <c r="E49" s="32" t="n"/>
+      <c r="F49" s="32" t="n"/>
+      <c r="G49" s="32" t="n"/>
+      <c r="H49" s="32" t="n"/>
+      <c r="I49" s="32" t="n"/>
+      <c r="J49" s="32" t="n"/>
+      <c r="K49" s="32" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>41B566322ACG1</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>TRAINLINE RESISTOR PANEL</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" t="n">
+        <v>2.859</v>
+      </c>
+      <c r="I50" t="n">
+        <v>2.859</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>14x6x8.5</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>85333990</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>41C663693G1</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>PANEL CPF</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>POWER</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" t="n">
+        <v>5.761</v>
+      </c>
+      <c r="I51" t="n">
+        <v>5.761</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>20.5x10.5x11.5</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>85371090</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>41A296352DNP57</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>REMOTE HEAD - VOICE RADIO RITRON</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Connectivity</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>VOICE RADIO</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>41A296326CYP77</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>M12-A_ MALE_ 8-PIN_ STRAIGHT BSH</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>16</v>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>41A296352PTP272</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>BC-PRECISION NAVIGATION MODULE</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>2</v>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>41A296352PTP58</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>AY-DISPLAY CSX PTC DISPLAY</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>41A296352PTP292</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>AX-POWER SUPPLY 13.6 V</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>1</v>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>MODEM ATT</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>MODEM ATT</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>3</v>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>84A237085AJP1</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>C-GoLIN EP_3 SMA_M2 CELL MODEM</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>1</v>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>17FL400B</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ST-DEVELOPER v19.4</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>1</v>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>41A296352CMP448</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>FB-DIGITAL RADIO MODULE</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>1</v>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>41A296352PTP326</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>BH-WABTEC TRAIN MANAGEMENT COMPUTER _WTMC_</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>1</v>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>17FM711C3</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>H-PANEL DBM</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>41A296352BCP9</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>N-HEAD OF TRAIN DEVICE</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>1</v>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>RL-1033772</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>ASSEMBLY, RELAY BOARD</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>1</v>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>41B549523ADP15</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>SWITCH PUSH BUTTON</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>2</v>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>BAP900F</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>CONVERTER/CHARGER DC/DC 74/72-F4WTSA</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>3</v>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>41A296352PTP360</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>_BB-CUT-OUT SWITCH CABINET</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>1</v>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>N265P21B</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>NUT, HEX, LOCK, 1/4-20, GR5, Z</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>1</v>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>N647AP21012B</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>BOLT, BHCS, 1/4"-20 X 3/4", 18-8</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>17</v>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1009634-901</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>SFM 701x Smart Fan Module</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>bottom on ACC</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>3</v>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>401581-100</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>SFPIM 703x 15v Smart Fan Module</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>41A296352VHP1_E-GEW</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>PTC-FILT-NB-160-MIL-U</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>160 MHz PTC Filter</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>later</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1</v>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>PTC-FILT-NB-220-MIL-MF</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>220 Mhz PTC FILTER</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>later</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>2</v>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>PTC Junction Box</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>1</v>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>41A296352LUP15</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>455 MHz Antenna (DPA, DPB, EOT )</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>SKID (Skid)</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>3</v>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>84D749224G1</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Power resistor</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Battery Skid?</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>1</v>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending; Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:M76">
+    <sortState ref="A2:M76">
+      <sortCondition descending="1" ref="F1"/>
+    </sortState>
+  </autoFilter>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Apply Harland's engineering weights, refresh Freight Handoff sheet
- Applied 19 engineering weights from Harland Updated Weigths.xlsx to
  Final Cost List (column W), overriding catalog/estimate values where
  they conflicted (TMC Panel, Air Brake Handle Assembly, LPS 17FH40),
  and filling the two remaining biggest unweighted items per Matheus:
  37495P (PTC Kit Master, ETMS Virgin Trains) = 100 lb and
  41A296352LUG24 (CSX Antenna Enclosure) = 300 lb.
- Marked all of these as "High" weight confidence with source
  "Engineering weight (Harland Updated Weights.xlsx)".
- Rebuilt Freight Handoff sheet from the refreshed weights and
  reapplied the AutoFilter on the header row.
</commit_message>
<xml_diff>
--- a/Lista_Final_Pathfinder_SKID_Custos_English_Updated.xlsx
+++ b/Lista_Final_Pathfinder_SKID_Custos_English_Updated.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="165" formatCode="\$\ #,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -100,6 +100,14 @@
       <color rgb="FF808080"/>
       <sz val="11"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF808080"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -155,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -213,6 +221,10 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1221,12 +1233,12 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>ESTIMATE (medium confidence) - Estimate from same-family PN 41A296352CMP433 (Distributed Power Module) - excludes the LXA radio portion - FLAGGED: Estimate covers only the DPM portion (same-family PN 41A296352CMP433) - excludes the LXA radio portion of this assembly. This is the single most expensive line item ($622k) - do not use this weight for freight without confirming with engineering.</t>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1285,6 +1297,19 @@
           <t>Direct supplier purchase; TP excluded; international freight 9%</t>
         </is>
       </c>
+      <c r="W3" t="n">
+        <v>45.359</v>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="35.25" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -1341,6 +1366,19 @@
           <t>TP included; international freight updated to 9%</t>
         </is>
       </c>
+      <c r="W4" t="n">
+        <v>1123.095</v>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="35.25" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
@@ -1397,6 +1435,19 @@
           <t>TP included; international freight updated to 9%</t>
         </is>
       </c>
+      <c r="W5" t="n">
+        <v>136.078</v>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="51.75" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -1453,6 +1504,19 @@
           <t>Direct supplier purchase; TP excluded; international freight 9%</t>
         </is>
       </c>
+      <c r="W6" t="n">
+        <v>134.263</v>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="35.25" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
@@ -1509,6 +1573,19 @@
           <t>Direct supplier purchase; TP excluded; international freight 9%</t>
         </is>
       </c>
+      <c r="W7" t="n">
+        <v>9.616</v>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="35.25" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -1565,6 +1642,19 @@
           <t>TP included; international freight updated to 9%</t>
         </is>
       </c>
+      <c r="W8" t="n">
+        <v>8.618</v>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="35.25" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
@@ -1642,6 +1732,19 @@
           <t>PAC/National is cheaper (by R$ 91,011.66)</t>
         </is>
       </c>
+      <c r="W9" t="n">
+        <v>2.268</v>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="35.25" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -1698,6 +1801,19 @@
           <t>TP included; international freight updated to 9%</t>
         </is>
       </c>
+      <c r="W10" t="n">
+        <v>9.071999999999999</v>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="35.25" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
@@ -1752,7 +1868,7 @@
         </is>
       </c>
       <c r="W11" t="n">
-        <v>27.216</v>
+        <v>20.412</v>
       </c>
       <c r="X11" t="inlineStr">
         <is>
@@ -1761,7 +1877,7 @@
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>Exact PN match in item catalog (17FL472A2)</t>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
@@ -1822,6 +1938,19 @@
           <t>TP included; international freight updated to 9%</t>
         </is>
       </c>
+      <c r="W12" t="n">
+        <v>25.855</v>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="35.25" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
@@ -1879,16 +2008,16 @@
         </is>
       </c>
       <c r="W13" t="n">
-        <v>29.03</v>
+        <v>7.938</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>ESTIMATE (medium confidence) - Estimate from same-PN-root 84A215295P73CCI4 (Fastbrake Brake Controller EVB)</t>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1947,6 +2076,19 @@
           <t>Direct supplier purchase; TP excluded; international freight 9%</t>
         </is>
       </c>
+      <c r="W14" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="35.25" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
@@ -2003,6 +2145,19 @@
           <t>TP included; international freight updated to 9%</t>
         </is>
       </c>
+      <c r="W15" t="n">
+        <v>7.575</v>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="35.25" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -2059,6 +2214,19 @@
           <t>Direct supplier purchase; TP excluded; international freight 9%</t>
         </is>
       </c>
+      <c r="W16" t="n">
+        <v>4.536</v>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="35.25" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
@@ -2113,7 +2281,7 @@
         </is>
       </c>
       <c r="W17" t="n">
-        <v>13.608</v>
+        <v>18.144</v>
       </c>
       <c r="X17" t="inlineStr">
         <is>
@@ -2127,7 +2295,7 @@
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>Exact PN match in item catalog (17FH40X1)</t>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
         </is>
       </c>
       <c r="AA17" t="inlineStr">
@@ -2267,6 +2435,19 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="W19" t="n">
+        <v>4.536</v>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="35.25" customHeight="1">
       <c r="B20" s="8" t="inlineStr">
@@ -2318,6 +2499,19 @@
           <t>Brazilian factory PAC price (local Brazilian cost)</t>
         </is>
       </c>
+      <c r="W20" t="n">
+        <v>2.268</v>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="35.25" customHeight="1">
       <c r="B21" s="8" t="inlineStr">
@@ -2367,6 +2561,19 @@
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>TP included; international freight updated to 9%</t>
+        </is>
+      </c>
+      <c r="W21" t="n">
+        <v>0.907</v>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>Engineering weight (Harland Updated Weights.xlsx)</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -14454,167 +14661,134 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="7"/>
-    <col width="13" customWidth="1" min="8" max="9"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="32" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1">
-      <c r="A1" s="30" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="33" t="inlineStr">
+        <is>
+          <t>US cost only - no Transfer Price, freight, or import duty applied. PAC-sourced items are excluded (their PAC price already includes TP + all freight + import duty).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="34" t="inlineStr">
         <is>
           <t>Part Number</t>
         </is>
       </c>
-      <c r="B1" s="30" t="inlineStr">
+      <c r="B2" s="34" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C1" s="30" t="inlineStr">
+      <c r="C2" s="34" t="inlineStr">
         <is>
           <t>System</t>
         </is>
       </c>
-      <c r="D1" s="30" t="inlineStr">
+      <c r="D2" s="34" t="inlineStr">
         <is>
           <t>SubSystem</t>
         </is>
       </c>
-      <c r="E1" s="30" t="inlineStr">
+      <c r="E2" s="34" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="F1" s="30" t="inlineStr">
+      <c r="F2" s="34" t="inlineStr">
         <is>
           <t>US Unit Cost (USD, no markup)</t>
         </is>
       </c>
-      <c r="G1" s="30" t="inlineStr">
+      <c r="G2" s="34" t="inlineStr">
         <is>
           <t>US Total Cost (USD, no markup)</t>
         </is>
       </c>
-      <c r="H1" s="30" t="inlineStr">
+      <c r="H2" s="34" t="inlineStr">
         <is>
           <t>Unit Weight (kg)</t>
         </is>
       </c>
-      <c r="I1" s="30" t="inlineStr">
+      <c r="I2" s="34" t="inlineStr">
         <is>
           <t>Total Weight (kg)</t>
         </is>
       </c>
-      <c r="J1" s="30" t="inlineStr">
+      <c r="J2" s="34" t="inlineStr">
         <is>
           <t>Dimensions (C x A x L, in)</t>
         </is>
       </c>
-      <c r="K1" s="30" t="inlineStr">
+      <c r="K2" s="34" t="inlineStr">
         <is>
           <t>NCM</t>
         </is>
       </c>
-      <c r="L1" s="30" t="inlineStr">
+      <c r="L2" s="34" t="inlineStr">
         <is>
           <t>Weight Confidence</t>
         </is>
       </c>
-      <c r="M1" s="30" t="inlineStr">
+      <c r="M2" s="34" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="31" t="inlineStr">
-        <is>
-          <t>41A296352CMP437</t>
-        </is>
-      </c>
-      <c r="B2" s="31" t="inlineStr">
-        <is>
-          <t>Dual Processor Module (DPM)+ LXA (Distributed Power Radio)</t>
-        </is>
-      </c>
-      <c r="C2" s="31" t="inlineStr">
-        <is>
-          <t>Controls (MCA, train control, er etc)</t>
-        </is>
-      </c>
-      <c r="D2" s="31" t="inlineStr">
-        <is>
-          <t>LXA</t>
-        </is>
-      </c>
-      <c r="E2" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="31" t="n">
-        <v>63100.8192</v>
-      </c>
-      <c r="G2" s="31" t="n">
-        <v>63100.8192</v>
-      </c>
-      <c r="H2" s="31" t="n">
-        <v>4.536</v>
-      </c>
-      <c r="I2" s="31" t="n">
-        <v>4.536</v>
-      </c>
-      <c r="J2" s="31" t="n"/>
-      <c r="K2" s="31" t="inlineStr">
-        <is>
-          <t>90328990</t>
-        </is>
-      </c>
-      <c r="L2" s="31" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="M2" s="31" t="inlineStr">
-        <is>
-          <t>FLAGGED - weight looks wrong, verify</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>41A296352LUG24</t>
+          <t>41A296352CMP437</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CSX Antenna Enclosure Arrangement</t>
+          <t>Dual Processor Module (DPM)+ LXA (Distributed Power Radio)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Connectivity</t>
+          <t>Controls (MCA, train control, er etc)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ANTENNA KIT Master</t>
+          <t>LXA</t>
         </is>
       </c>
       <c r="E3" t="n">
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>30000</v>
+        <v>63100.8192</v>
       </c>
       <c r="G3" t="n">
-        <v>30000</v>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>63100.8192</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4.536</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4.536</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>90328990</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -14648,165 +14822,195 @@
       <c r="G4" t="n">
         <v>28529</v>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+      <c r="H4" t="n">
+        <v>45.359</v>
+      </c>
+      <c r="I4" t="n">
+        <v>45.359</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>84A215295P62</t>
+          <t>84A222059P5</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Pneumatic Brake Control System (Including lament and control portions) Includes EM EAB Control Functionality</t>
+          <t>BATTERIES</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Fastbrake</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>23409.1</v>
+        <v>15685.42</v>
       </c>
       <c r="G5" t="n">
-        <v>23409.1</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>31370.84</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1123.095</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2246.19</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>41A296352DNP37</t>
+          <t>41A296352LUG24</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>RADIO PRAD PTC RADIO</t>
+          <t>CSX Antenna Enclosure Arrangement</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>Connectivity</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>ANTENNA KIT Master</t>
         </is>
       </c>
       <c r="E6" t="n">
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>20000</v>
+        <v>30000</v>
       </c>
       <c r="G6" t="n">
-        <v>20000</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>30000</v>
+      </c>
+      <c r="H6" t="n">
+        <v>136.078</v>
+      </c>
+      <c r="I6" t="n">
+        <v>136.078</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>84A222059P5</t>
+          <t>84A215295P62</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BATTERIES</t>
+          <t>Pneumatic Brake Control System (Including lament and control portions) Includes EM EAB Control Functionality</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Air</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>POWER</t>
+          <t>Fastbrake</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>15685.42</v>
+        <v>23409.1</v>
       </c>
       <c r="G7" t="n">
-        <v>31370.84</v>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>23409.1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>134.263</v>
+      </c>
+      <c r="I7" t="n">
+        <v>134.263</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>84A237085AEP121</t>
+          <t>41A296352DNP37</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8 Slot ACC Chassis for MCA w/ i7 HPEAP and SMM2 Cards</t>
+          <t>RADIO PRAD PTC RADIO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Controls (MCA, train control, er etc)</t>
+          <t>PTC</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>TRAIN CONTROL</t>
+          <t>PTC</t>
         </is>
       </c>
       <c r="E8" t="n">
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>8000</v>
+        <v>20000</v>
       </c>
       <c r="G8" t="n">
-        <v>8000</v>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>20000</v>
+      </c>
+      <c r="H8" t="n">
+        <v>9.616</v>
+      </c>
+      <c r="I8" t="n">
+        <v>9.616</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>17KC108E28</t>
+          <t>17FM878A6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MASTER CONTROLLER</t>
+          <t>NIO 2.0</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -14816,80 +15020,81 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>TRAIN CONTROL</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>5877.102</v>
+        <v>5176.9118</v>
       </c>
       <c r="G9" t="n">
-        <v>5877.102</v>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>15530.7354</v>
+      </c>
+      <c r="H9" t="n">
+        <v>8.618</v>
+      </c>
+      <c r="I9" t="n">
+        <v>25.854</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>84A215295P73</t>
+          <t>L7000083-900</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Air Brake Handle Assembly (AAR Console)</t>
+          <t>Wireless Communications Management Module, Gen 3 (WCM3)​</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Controls (MCA, train control, er etc)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Fastbrake</t>
+          <t>TRAIN CONTROL</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
-        <v>5702.83</v>
+        <v>5000</v>
       </c>
       <c r="G10" t="n">
-        <v>5702.83</v>
+        <v>10000</v>
       </c>
       <c r="H10" t="n">
-        <v>29.03</v>
+        <v>2.268</v>
       </c>
       <c r="I10" t="n">
-        <v>29.03</v>
+        <v>4.536</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Weight is an estimate (similar item)</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>17FM878A6</t>
+          <t>84A237085AEP121</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NIO 2.0</t>
+          <t>8 Slot ACC Chassis for MCA w/ i7 HPEAP and SMM2 Cards</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -14899,33 +15104,39 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>TRAIN CONTROL</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>5176.9118</v>
+        <v>8000</v>
       </c>
       <c r="G11" t="n">
-        <v>15530.7354</v>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>8000</v>
+      </c>
+      <c r="H11" t="n">
+        <v>9.071999999999999</v>
+      </c>
+      <c r="I11" t="n">
+        <v>9.071999999999999</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>L7000083-900</t>
+          <t>17KC108E28</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Wireless Communications Management Module, Gen 3 (WCM3)​</t>
+          <t>MASTER CONTROLLER</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -14939,161 +15150,191 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>5000</v>
+        <v>5877.102</v>
       </c>
       <c r="G12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>5877.102</v>
+      </c>
+      <c r="H12" t="n">
+        <v>25.855</v>
+      </c>
+      <c r="I12" t="n">
+        <v>25.855</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>17FM868B2</t>
+          <t>84A215295P73</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SNIO</t>
+          <t>Air Brake Handle Assembly (AAR Console)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Controls (MCA, train control, er etc)</t>
+          <t>Air</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>Fastbrake</t>
         </is>
       </c>
       <c r="E13" t="n">
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>4150.9559</v>
+        <v>5702.83</v>
       </c>
       <c r="G13" t="n">
-        <v>4150.9559</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>5702.83</v>
+      </c>
+      <c r="H13" t="n">
+        <v>7.938</v>
+      </c>
+      <c r="I13" t="n">
+        <v>7.938</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>41A296352DNP55</t>
+          <t>17FM868B2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>VOICE RADIO RITRON</t>
+          <t>SNIO</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Connectivity</t>
+          <t>Controls (MCA, train control, er etc)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>VOICE RADIO</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="E14" t="n">
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>3933</v>
+        <v>4150.9559</v>
       </c>
       <c r="G14" t="n">
-        <v>3933</v>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>4150.9559</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="I14" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>32613P</t>
+          <t>41A296352DNP55</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>KIT ETMS AXLE INTERFACE FOR WPart Number 29266P</t>
+          <t>VOICE RADIO RITRON</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>Connectivity</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>VOICE RADIO</t>
         </is>
       </c>
       <c r="E15" t="n">
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>2981.71</v>
+        <v>3933</v>
       </c>
       <c r="G15" t="n">
-        <v>2981.71</v>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>3933</v>
+      </c>
+      <c r="H15" t="n">
+        <v>7.575</v>
+      </c>
+      <c r="I15" t="n">
+        <v>7.575</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>41B546155P2</t>
+          <t>32613P</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Horn</t>
+          <t>KIT ETMS AXLE INTERFACE FOR WPart Number 29266P</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Controls (MCA, train control, er etc)</t>
+          <t>PTC</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>TRAIN CONTROL</t>
+          <t>PTC</t>
         </is>
       </c>
       <c r="E16" t="n">
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>1891.99</v>
+        <v>2981.71</v>
       </c>
       <c r="G16" t="n">
-        <v>1891.99</v>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>2981.71</v>
+      </c>
+      <c r="H16" t="n">
+        <v>4.536</v>
+      </c>
+      <c r="I16" t="n">
+        <v>4.536</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -15152,47 +15393,42 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>84A215295P3</t>
+          <t>41B546155P2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>POU-to-Handle cable 18' length</t>
+          <t>Horn</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Controls (MCA, train control, er etc)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Fastbrake</t>
+          <t>TRAIN CONTROL</t>
         </is>
       </c>
       <c r="E18" t="n">
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>1036.89</v>
+        <v>1891.99</v>
       </c>
       <c r="G18" t="n">
-        <v>1036.89</v>
+        <v>1891.99</v>
       </c>
       <c r="H18" t="n">
-        <v>1.247</v>
+        <v>4.536</v>
       </c>
       <c r="I18" t="n">
-        <v>1.247</v>
+        <v>4.536</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>Weight is an estimate (similar item)</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -15221,166 +15457,183 @@
       <c r="G19" t="n">
         <v>1600</v>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+      <c r="H19" t="n">
+        <v>2.268</v>
+      </c>
+      <c r="I19" t="n">
+        <v>4.536</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>LED Ditch Light</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>TRAIN CONTROL</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" t="n">
+        <v>375</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.907</v>
+      </c>
+      <c r="I20" t="n">
+        <v>3.628</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>84A215295P3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>POU-to-Handle cable 18' length</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Fastbrake</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1036.89</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1036.89</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1.247</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1.247</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Weight is an estimate (similar item)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>41B566322ACG1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TRAINLINE RESISTOR PANEL</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>SKID Assembly</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2.859</v>
+      </c>
+      <c r="I22" t="n">
+        <v>2.859</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>14x6x8.5</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>85333990</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>No US cost yet - price pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>RCCR-RMTCBL-RA-CUSTOM</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>VOICE RADIO RITRON CABLE,REMOTE,RR-225/XXX, RCCR,RIGHT
 ANGLE,19-PIN,FLAME RETARDANT</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Connectivity</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>VOICE RADIO</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" t="n">
-        <v>761</v>
-      </c>
-      <c r="G20" t="n">
-        <v>761</v>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>41A296352PTP306/41A296352PTP122</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Assembled Air Manifold (Contains 3 pressure sensors mounted in appropriate locations on Air Manifold.)</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>PTC</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>PTC</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" t="n">
-        <v>595.7889</v>
-      </c>
-      <c r="G21" t="n">
-        <v>595.7889</v>
-      </c>
-      <c r="H21" t="n">
-        <v>5.897</v>
-      </c>
-      <c r="I21" t="n">
-        <v>5.897</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>85381000</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>Weight is an estimate (similar item)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>32447P</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>ASY CABLE WHEEL TACH AC EVO/SD70 ACE</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>PTC</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>PTC</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" t="n">
-        <v>411.22</v>
-      </c>
-      <c r="G22" t="n">
-        <v>411.22</v>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>41A296352PTP10/319/34</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>VALVE Part NumberEUMATIC NC/CO (Penalty Magnet Valve) Graham-White 812-142</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>PTC</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>PTC</t>
         </is>
       </c>
       <c r="E23" t="n">
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>404.6239</v>
+        <v>761</v>
       </c>
       <c r="G23" t="n">
-        <v>404.6239</v>
+        <v>761</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -15389,45 +15642,65 @@
       </c>
     </row>
     <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>41C663693G1</t>
+        </is>
+      </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>LED Ditch Light</t>
+          <t>PANEL CPF</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Controls (MCA, train control, er etc)</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>TRAIN CONTROL</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
-      </c>
-      <c r="F24" t="n">
-        <v>375</v>
-      </c>
-      <c r="G24" t="n">
-        <v>1500</v>
+        <v>1</v>
+      </c>
+      <c r="H24" t="n">
+        <v>5.761</v>
+      </c>
+      <c r="I24" t="n">
+        <v>5.761</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>20.5x10.5x11.5</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>85371090</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Weight not found - needs supplier data</t>
+          <t>No US cost yet - price pending</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>84A231123CSP30</t>
+          <t>41A296352PTP306/41A296352PTP122</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Axle Tac - WRE Part Number: 29266P</t>
+          <t>Assembled Air Manifold (Contains 3 pressure sensors mounted in appropriate locations on Air Manifold.)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -15444,46 +15717,62 @@
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>205</v>
+        <v>595.7889</v>
       </c>
       <c r="G25" t="n">
-        <v>205</v>
+        <v>595.7889</v>
+      </c>
+      <c r="H25" t="n">
+        <v>5.897</v>
+      </c>
+      <c r="I25" t="n">
+        <v>5.897</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>85381000</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Weight not found - needs supplier data</t>
+          <t>Weight is an estimate (similar item)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>84A201850P4</t>
+          <t>32447P</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ENGINE CONTROL SWITCH</t>
+          <t>ASY CABLE WHEEL TACH AC EVO/SD70 ACE</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Controls (MCA, train control, er etc)</t>
+          <t>PTC</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>TRAIN CONTROL</t>
+          <t>PTC</t>
         </is>
       </c>
       <c r="E26" t="n">
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>171.544</v>
+        <v>411.22</v>
       </c>
       <c r="G26" t="n">
-        <v>171.544</v>
+        <v>411.22</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -15494,32 +15783,32 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>RCCR-PWRCBL</t>
+          <t>41A296352PTP10/319/34</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CABLE, PWR, 72V,RA,6.5FT (78").,RR-070,RCCR</t>
+          <t>VALVE Part NumberEUMATIC NC/CO (Penalty Magnet Valve) Graham-White 812-142</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Connectivity</t>
+          <t>PTC</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>VOICE RADIO</t>
+          <t>PTC</t>
         </is>
       </c>
       <c r="E27" t="n">
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>159</v>
+        <v>404.6239</v>
       </c>
       <c r="G27" t="n">
-        <v>159</v>
+        <v>404.6239</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -15530,32 +15819,32 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>17 pin MS3106-20-29F</t>
+          <t>84A231123CSP30</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Head of Train Device - Padom - J2 Connector</t>
+          <t>Axle Tac - WRE Part Number: 29266P</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Controls (MCA, train control, er etc)</t>
+          <t>PTC</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Wiring</t>
+          <t>PTC</t>
         </is>
       </c>
       <c r="E28" t="n">
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>79.83</v>
+        <v>205</v>
       </c>
       <c r="G28" t="n">
-        <v>79.83</v>
+        <v>205</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
@@ -15566,12 +15855,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5088-7000-P4611-0000000-ND‎</t>
+          <t>84A207079ABP1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>POE Power Connector on SMM2 (M12 FEMALE 0 L-CODED FIELD-WIREA)</t>
+          <t>41A313392DCP18 alternative 300" /</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -15581,33 +15870,49 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>TRAIN CONTROL</t>
+          <t>Wiring</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="F29" t="n">
-        <v>72.41</v>
+        <v>8.118</v>
       </c>
       <c r="G29" t="n">
-        <v>72.41</v>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>202.95</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.227</v>
+      </c>
+      <c r="I29" t="n">
+        <v>5.675</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>24x20x24</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>85446000</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>41A296352PTP67</t>
+          <t>84A201850P4</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CABLE CSX 12V P WR CBL</t>
+          <t>ENGINE CONTROL SWITCH</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -15617,17 +15922,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>TRAIN CONTROL</t>
         </is>
       </c>
       <c r="E30" t="n">
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>71.94</v>
+        <v>171.544</v>
       </c>
       <c r="G30" t="n">
-        <v>71.94</v>
+        <v>171.544</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
@@ -15638,32 +15943,32 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>41A296352PTP69</t>
+          <t>RCCR-PWRCBL</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CABLE CSX 74V P WR CBL</t>
+          <t>CABLE, PWR, 72V,RA,6.5FT (78").,RR-070,RCCR</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Controls (MCA, train control, er etc)</t>
+          <t>Connectivity</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>VOICE RADIO</t>
         </is>
       </c>
       <c r="E31" t="n">
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>71.94</v>
+        <v>159</v>
       </c>
       <c r="G31" t="n">
-        <v>71.94</v>
+        <v>159</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
@@ -15674,650 +15979,618 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>16246P</t>
+          <t>41A216641AMP126</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Flexi-Axle - WRE Part Number: 16246P</t>
+          <t>NIO1D CONNECTOR BACKSHELL</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>Controls (MCA, train control, er etc)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>Wiring</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F32" t="n">
-        <v>59.75</v>
+        <v>29.9096</v>
       </c>
       <c r="G32" t="n">
-        <v>59.75</v>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>89.72880000000001</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>0x0x0</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>17 pin MS3106-20-29F</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Head of Train Device - Padom - J2 Connector</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>79.83</v>
+      </c>
+      <c r="G33" t="n">
+        <v>79.83</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>41A216641AMP125</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>NIO1A CONNECTOR BACKSHELL</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>3</v>
+      </c>
+      <c r="F34" t="n">
+        <v>24.1998</v>
+      </c>
+      <c r="G34" t="n">
+        <v>72.5994</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>0x0x0</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>5088-7000-P4611-0000000-ND‎</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>POE Power Connector on SMM2 (M12 FEMALE 0 L-CODED FIELD-WIREA)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>TRAIN CONTROL</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>72.41</v>
+      </c>
+      <c r="G35" t="n">
+        <v>72.41</v>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>41A296352PTP67</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>CABLE CSX 12V P WR CBL</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>MCA</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" t="n">
+        <v>71.94</v>
+      </c>
+      <c r="G36" t="n">
+        <v>71.94</v>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>41A296352PTP69</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>CABLE CSX 74V P WR CBL</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>MCA</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="n">
+        <v>71.94</v>
+      </c>
+      <c r="G37" t="n">
+        <v>71.94</v>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>41A216641AMP93</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>NIO1E CONNECTOR</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" t="n">
+        <v>23.9499</v>
+      </c>
+      <c r="G38" t="n">
+        <v>71.8497</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.162</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>0x0x0</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>41A216641AMP103</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>NIO1D CONNECTOR</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>3</v>
+      </c>
+      <c r="F39" t="n">
+        <v>21.2198</v>
+      </c>
+      <c r="G39" t="n">
+        <v>63.6594</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>1.5x1x1.5</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>16246P</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Flexi-Axle - WRE Part Number: 16246P</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" t="n">
+        <v>59.75</v>
+      </c>
+      <c r="G40" t="n">
+        <v>59.75</v>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>41A216641AMP99</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>NIO1B CONNECTOR</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" t="n">
+        <v>19.67</v>
+      </c>
+      <c r="G41" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>0x0x0</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>41A216641AMP123</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>NIO1F CONNECTOR BACKSHELL</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" t="n">
+        <v>19.5574</v>
+      </c>
+      <c r="G42" t="n">
+        <v>58.6722</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>0x0x0</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>41A216641AMP100</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>NIO1C CONNECTOR</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" t="n">
+        <v>19.173</v>
+      </c>
+      <c r="G43" t="n">
+        <v>57.519</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>0x0x0</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>41A216641AMP86</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>NIO1F CONNECTOR</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>3</v>
+      </c>
+      <c r="F44" t="n">
+        <v>18.9357</v>
+      </c>
+      <c r="G44" t="n">
+        <v>56.8071</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>3.95x1.25x6.65</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>41A216641AMP98</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>NIO1A CONNECTOR</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" t="n">
+        <v>15.455</v>
+      </c>
+      <c r="G45" t="n">
+        <v>46.365</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0.159</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>0x0x0</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>41A216641ABP153</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>HELPER'S RADIO SPEAKER 
 CONNECTOR</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Controls (MCA, train control, er etc)</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Wiring</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" t="n">
-        <v>45.7356</v>
-      </c>
-      <c r="G33" t="n">
-        <v>45.7356</v>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>41A216641AMP126</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>NIO1D CONNECTOR BACKSHELL</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Controls (MCA, train control, er etc)</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Wiring</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>3</v>
-      </c>
-      <c r="F34" t="n">
-        <v>29.9096</v>
-      </c>
-      <c r="G34" t="n">
-        <v>89.72880000000001</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>0x0x0</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>41A216641AMP125</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>NIO1A CONNECTOR BACKSHELL</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Controls (MCA, train control, er etc)</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Wiring</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>3</v>
-      </c>
-      <c r="F35" t="n">
-        <v>24.1998</v>
-      </c>
-      <c r="G35" t="n">
-        <v>72.5994</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="I35" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>0x0x0</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>41A216641AMP93</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>NIO1E CONNECTOR</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Controls (MCA, train control, er etc)</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Wiring</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>3</v>
-      </c>
-      <c r="F36" t="n">
-        <v>23.9499</v>
-      </c>
-      <c r="G36" t="n">
-        <v>71.8497</v>
-      </c>
-      <c r="H36" t="n">
-        <v>0.054</v>
-      </c>
-      <c r="I36" t="n">
-        <v>0.162</v>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>0x0x0</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>41A212414P31, 41A212414P3 2-Pole Option</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>AUTOCOUPLER CIRCUIT BREAKER,  CCB(2A)</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Controls (MCA, train control, er etc)</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Circuit Breaker</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" t="n">
-        <v>22.0206</v>
-      </c>
-      <c r="G37" t="n">
-        <v>22.0206</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="I37" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>2.5x0.65x3.05</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>85362000</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>41A216641AMP103</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>NIO1D CONNECTOR</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Controls (MCA, train control, er etc)</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Wiring</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>3</v>
-      </c>
-      <c r="F38" t="n">
-        <v>21.2198</v>
-      </c>
-      <c r="G38" t="n">
-        <v>63.6594</v>
-      </c>
-      <c r="H38" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="I38" t="n">
-        <v>0.135</v>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>1.5x1x1.5</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>41A216641AMP99</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>NIO1B CONNECTOR</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Controls (MCA, train control, er etc)</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Wiring</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>3</v>
-      </c>
-      <c r="F39" t="n">
-        <v>19.67</v>
-      </c>
-      <c r="G39" t="n">
-        <v>59.01</v>
-      </c>
-      <c r="H39" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>0x0x0</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>41A216641AMP123</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>NIO1F CONNECTOR BACKSHELL</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Controls (MCA, train control, er etc)</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Wiring</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>3</v>
-      </c>
-      <c r="F40" t="n">
-        <v>19.5574</v>
-      </c>
-      <c r="G40" t="n">
-        <v>58.6722</v>
-      </c>
-      <c r="H40" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="I40" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>0x0x0</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>41A216641AMP100</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>NIO1C CONNECTOR</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Controls (MCA, train control, er etc)</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Wiring</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>3</v>
-      </c>
-      <c r="F41" t="n">
-        <v>19.173</v>
-      </c>
-      <c r="G41" t="n">
-        <v>57.519</v>
-      </c>
-      <c r="H41" t="n">
-        <v>0</v>
-      </c>
-      <c r="I41" t="n">
-        <v>0</v>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>0x0x0</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>41A216641AMP86</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>NIO1F CONNECTOR</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Controls (MCA, train control, er etc)</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Wiring</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>3</v>
-      </c>
-      <c r="F42" t="n">
-        <v>18.9357</v>
-      </c>
-      <c r="G42" t="n">
-        <v>56.8071</v>
-      </c>
-      <c r="H42" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="I42" t="n">
-        <v>0.096</v>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>3.95x1.25x6.65</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>41A216641AMP98</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>NIO1A CONNECTOR</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Controls (MCA, train control, er etc)</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Wiring</t>
-        </is>
-      </c>
-      <c r="E43" t="n">
-        <v>3</v>
-      </c>
-      <c r="F43" t="n">
-        <v>15.455</v>
-      </c>
-      <c r="G43" t="n">
-        <v>46.365</v>
-      </c>
-      <c r="H43" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="I43" t="n">
-        <v>0.159</v>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>0x0x0</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>5373-219</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>CONNECTOR, ELECTRICAL</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Controls (MCA, train control, er etc)</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Wiring</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>1</v>
-      </c>
-      <c r="F44" t="n">
-        <v>13.66</v>
-      </c>
-      <c r="G44" t="n">
-        <v>13.66</v>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>84A207079ABP1</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>41A313392DCP18 alternative 300" /</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Controls (MCA, train control, er etc)</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Wiring</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
-        <v>25</v>
-      </c>
-      <c r="F45" t="n">
-        <v>8.118</v>
-      </c>
-      <c r="G45" t="n">
-        <v>202.95</v>
-      </c>
-      <c r="H45" t="n">
-        <v>0.227</v>
-      </c>
-      <c r="I45" t="n">
-        <v>5.675</v>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>24x20x24</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>85446000</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>41A271471P24/38</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>HPEAP DISCRETE CONNECTOR Backshell</t>
-        </is>
-      </c>
       <c r="C46" t="inlineStr">
         <is>
           <t>Controls (MCA, train control, er etc)</t>
@@ -16332,42 +16605,26 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>1.9294</v>
+        <v>45.7356</v>
       </c>
       <c r="G46" t="n">
-        <v>1.9294</v>
-      </c>
-      <c r="H46" t="n">
-        <v>0.023</v>
-      </c>
-      <c r="I46" t="n">
-        <v>0.023</v>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>5.1x1.15x2.95</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>85366990</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>45.7356</v>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Weight not found - needs supplier data</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>41A296352DNP73</t>
+          <t>41A212414P31, 41A212414P3 2-Pole Option</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CABLE: GROUND S TRAP</t>
+          <t>AUTOCOUPLER CIRCUIT BREAKER,  CCB(2A)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -16377,33 +16634,49 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>Circuit Breaker</t>
         </is>
       </c>
       <c r="E47" t="n">
         <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>0.01</v>
+        <v>22.0206</v>
       </c>
       <c r="G47" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>Weight not found - needs supplier data</t>
+        <v>22.0206</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.093</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0.093</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2.5x0.65x3.05</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>85362000</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>41A296352DNP96</t>
+          <t>5373-219</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Cable: CRM Ethernet Switch to ACC</t>
+          <t>CONNECTOR, ELECTRICAL</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -16413,17 +16686,17 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>Wiring</t>
         </is>
       </c>
       <c r="E48" t="n">
         <v>1</v>
       </c>
       <c r="F48" t="n">
-        <v>0.01</v>
+        <v>13.66</v>
       </c>
       <c r="G48" t="n">
-        <v>0.01</v>
+        <v>13.66</v>
       </c>
       <c r="M48" t="inlineStr">
         <is>
@@ -16432,121 +16705,126 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="32" t="inlineStr">
-        <is>
-          <t>US cost only - no Transfer Price, freight, or import duty applied. PAC-sourced items are excluded (their PAC price already includes TP + all freight + import duty).</t>
-        </is>
-      </c>
-      <c r="B49" s="32" t="n"/>
-      <c r="C49" s="32" t="n"/>
-      <c r="D49" s="32" t="n"/>
-      <c r="E49" s="32" t="n"/>
-      <c r="F49" s="32" t="n"/>
-      <c r="G49" s="32" t="n"/>
-      <c r="H49" s="32" t="n"/>
-      <c r="I49" s="32" t="n"/>
-      <c r="J49" s="32" t="n"/>
-      <c r="K49" s="32" t="n"/>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>41A271471P24/38</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>HPEAP DISCRETE CONNECTOR Backshell</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Controls (MCA, train control, er etc)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" t="n">
+        <v>1.9294</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1.9294</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>5.1x1.15x2.95</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>85366990</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>41B566322ACG1</t>
+          <t>41A296352DNP73</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TRAINLINE RESISTOR PANEL</t>
+          <t>CABLE: GROUND S TRAP</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>SKID Assembly</t>
+          <t>Controls (MCA, train control, er etc)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Controls (MCA, train control, er etc)</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="E50" t="n">
         <v>1</v>
       </c>
-      <c r="H50" t="n">
-        <v>2.859</v>
-      </c>
-      <c r="I50" t="n">
-        <v>2.859</v>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>14x6x8.5</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>85333990</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+      <c r="F50" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0.01</v>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>No US cost yet - price pending</t>
+          <t>Weight not found - needs supplier data</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>41C663693G1</t>
+          <t>41A296352DNP96</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PANEL CPF</t>
+          <t>Cable: CRM Ethernet Switch to ACC</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Controls (MCA, train control, er etc)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>POWER</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="E51" t="n">
         <v>1</v>
       </c>
-      <c r="H51" t="n">
-        <v>5.761</v>
-      </c>
-      <c r="I51" t="n">
-        <v>5.761</v>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>20.5x10.5x11.5</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>85371090</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+      <c r="F51" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.01</v>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>No US cost yet - price pending</t>
+          <t>Weight not found - needs supplier data</t>
         </is>
       </c>
     </row>
@@ -17296,11 +17574,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:M76">
-    <sortState ref="A2:M76">
-      <sortCondition descending="1" ref="F1"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A2:M76"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add P&L Pathfinder sheet with real pricing methodology (TP/TDM/NCM)
- New "P&L Pathfinder" sheet implements the verified Material Pricing /
  Approval Summary cascade: TP is WBT USA's own margin (feeds Frete
  Intl/II like a real cost, but is excluded from WBT Brazil's own
  margin base per Total Deal Margin = (TP + GM BRZ) / Preco Liquido);
  P&L Old was discarded (its formulas are broken/#REF!).
- Uses real China Gate freight quote (Frete Intl 1.23%, Frete Nacional
  flat R$21,753.10) instead of the old 9%/3% assumptions, and FX 5.10
  from Material Pricing's own RATES tab.
- II/IPI/PIS-COFINS use real per-NCM rates (from Material Pricing's
  "II" tab) for the 6 priced imported items with a confirmed NCM;
  worst-case flat rates for the other 41 without one.
- Editable Cambio, TDM, and tax-rate cells drive live formulas down to
  both headline numbers: "Nosso Preco" (cost + margin, business view)
  and "Preco Final ao Cliente" (all taxes included, client ROI view).
</commit_message>
<xml_diff>
--- a/Lista_Final_Pathfinder_SKID_Custos_English_Updated.xlsx
+++ b/Lista_Final_Pathfinder_SKID_Custos_English_Updated.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDT Integration and Assembly" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missing Items" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Freight Handoff" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;L Pathfinder" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Final Cost List'!$A$1:$O$165</definedName>
@@ -27,7 +28,7 @@
     <numFmt numFmtId="165" formatCode="\$\ #,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -108,6 +109,26 @@
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF808080"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -129,7 +150,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -159,11 +180,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -225,6 +260,16 @@
     <xf numFmtId="0" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="16" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -17580,4 +17625,333 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="35" t="inlineStr">
+        <is>
+          <t>P&amp;L PATHFINDER - PREÇO REAL (metodologia Material Pricing / Approval Summary)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Câmbio (USD-&gt;BRL):</t>
+        </is>
+      </c>
+      <c r="B3" s="36" t="n">
+        <v>5.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Total Deal Margin (TDM):</t>
+        </is>
+      </c>
+      <c r="B4" s="37" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C4" s="38" t="inlineStr">
+        <is>
+          <t>&lt;- editável. Ajusta o Preço Líquido e o Preço ao Cliente automaticamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PIS/COFINS (blended, NCM real onde disponível):</t>
+        </is>
+      </c>
+      <c r="B5" s="39" t="n">
+        <v>0.1006</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ICMS:</t>
+        </is>
+      </c>
+      <c r="B6" s="39" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IPI (blended, NCM real onde disponível):</t>
+        </is>
+      </c>
+      <c r="B7" s="39" t="n">
+        <v>0.0969</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="40" t="inlineStr">
+        <is>
+          <t>1) CUSTO (Raw Cost + TP + Frete + II)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Raw Cost - Itens Importados (BOM USD x Qtd x Câmbio)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>1346980.92</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Raw Cost - Itens PAC (já nacionalizado, all-in local)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>166060.16</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TP - Transfer Price (13%/17,2% conforme grupo; é a margem da WBT USA)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>198163.69</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Frete Internacional (real, cotação China Gate, 1,23%)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>18998.55</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>II - Imposto de Importação (blended 17.96%, NCM real onde disponível)</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>280915.82</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Frete Nacional (real, cotação China Gate, Santos-&gt;Betim/Contagem)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>21753.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="41">
+        <f> CUSTO FINAL (com TP)</f>
+        <v/>
+      </c>
+      <c r="B16" s="42">
+        <f>SUM(B10:B15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="40" t="inlineStr">
+        <is>
+          <t>2) MARGEM (TDM aplicado sobre o custo SEM o TP; TP é devolvido depois sem markup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Base p/ margem (Custo Final - TP)</t>
+        </is>
+      </c>
+      <c r="B19" s="3">
+        <f>B16-B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Preço Líquido s/ TP (Base / (1 - TDM))</t>
+        </is>
+      </c>
+      <c r="B20" s="3">
+        <f>B19/(1-$B$4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="41">
+        <f> PREÇO LÍQUIDO ('NOSSO PREÇO' - custo + margem, sem impostos de saída)</f>
+        <v/>
+      </c>
+      <c r="B21" s="42">
+        <f>B20+B12</f>
+        <v/>
+      </c>
+      <c r="C21" s="43">
+        <f>B21/$B$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="40" t="inlineStr">
+        <is>
+          <t>3) IMPOSTOS DE SAÍDA (não afetam nossa margem - o cliente paga, cliente pode creditar parte)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>+ PIS/COFINS (por dentro)</t>
+        </is>
+      </c>
+      <c r="B24" s="3">
+        <f>B21/(1-$B$5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>+ ICMS (por dentro, empilhado sobre PIS/COFINS)</t>
+        </is>
+      </c>
+      <c r="B25" s="3">
+        <f>B24/(1-$B$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>+ IPI (por fora, % sobre o valor já com ICMS)</t>
+        </is>
+      </c>
+      <c r="B26" s="3">
+        <f>B25*$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="41">
+        <f> PREÇO FINAL AO CLIENTE (com todos os impostos)</f>
+        <v/>
+      </c>
+      <c r="B27" s="42">
+        <f>B25+B26</f>
+        <v/>
+      </c>
+      <c r="C27" s="43">
+        <f>B27/$B$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="44" t="inlineStr">
+        <is>
+          <t>Notas / Premissas:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="38" t="inlineStr">
+        <is>
+          <t>- Metodologia: aba 'Material Pricing' + 'Approval Summary' do Material Pricing.xlsm (P&amp;L Old descartado - fórmulas quebradas/#REF!).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="38" t="inlineStr">
+        <is>
+          <t>- TP tratado como a margem da WBT USA (GM WBT USA); entra no custo mas fica fora da base de margem da WBT Brasil (TDM = (TP + GM BRZ) / Preço Líquido).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="38" t="inlineStr">
+        <is>
+          <t>- Frete Internacional e Frete Nacional: valores reais da cotação China Gate (Planilha de Custos de Importação - Pathfinder - Set 26.xlsx), não os 9%/3% antigos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="38" t="inlineStr">
+        <is>
+          <t>- II/IPI/PIS-COFINS: taxa real por NCM (aba 'II' do Material Pricing) para os 6 itens com NCM confirmado; taxa 'pior caso' (nossa antiga flat) para os demais 41 itens importados sem NCM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="38" t="inlineStr">
+        <is>
+          <t>- ICMS: 18% flat (mesmo valor usado no exemplo real da Material Pricing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="38" t="inlineStr">
+        <is>
+          <t>- 88 itens PAC somados como um bloco só (já é custo all-in local, sem decompor TP/frete/II).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="38" t="inlineStr">
+        <is>
+          <t>- 27 itens ainda sem cotação de custo (Missing) NÃO estão incluídos neste total - ver aba 'Missing Items'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="38" t="inlineStr">
+        <is>
+          <t>- QQP (tributos de serviço) e ISS (imposto do rollup GDT de integração/labor) foram desconsiderados por enquanto, a pedido.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A30:F30"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Price Calculation Detail tab with sources for every number
- New "Detalhamento do Preço" / "Price Calc Detail" tab in all three
  workbooks, so every line in the P&L can be traced back to its
  source (Material Pricing.xlsm, the China Gate freight quote, the
  Final Cost List, etc.) instead of just showing a result to question.
- Includes a Reality Check section: Our Price (Net, before Brazilian
  taxes) is US$945,272 - close to the US$900k domestic reference -
  while the Final Client Price (US$1,405,909) is inflated entirely by
  Brazilian import duty and consumption taxes (II/IPI/PIS/COFINS/ICMS),
  which don't exist in a US domestic sale and would apply the same way
  whether importing components or a finished railcar.
- Full waterfall with formula/logic and source citation per line, an
  assumptions register (value used, confidence, where it could be
  wrong), and a margin sensitivity table (30%-55% TDM).
</commit_message>
<xml_diff>
--- a/Lista_Final_Pathfinder_SKID_Custos_English_Updated.xlsx
+++ b/Lista_Final_Pathfinder_SKID_Custos_English_Updated.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missing Items" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Freight Handoff" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;L Pathfinder" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalhamento do Preço" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Final Cost List'!$A$1:$O$165</definedName>
@@ -130,7 +131,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -147,6 +148,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -198,7 +205,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -270,6 +277,12 @@
     <xf numFmtId="164" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="16" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="19" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -17975,4 +17988,948 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F68"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="35" t="inlineStr">
+        <is>
+          <t>DETALHAMENTO DO CÁLCULO DE PREÇO - origem e fórmula de cada número</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="38" t="inlineStr">
+        <is>
+          <t>Use esta aba pra responder 'por que esse número é X' - cada linha cita a fonte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="41" t="inlineStr">
+        <is>
+          <t>0) CHECAGEM DE REALIDADE vs. preço doméstico nos EUA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Preço de Referência Doméstico EUA (input - digite o valor real aqui):</t>
+        </is>
+      </c>
+      <c r="B5" s="45" t="n">
+        <v>900000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Nosso Preço (Líquido - custo + margem, antes dos impostos brasileiros de saída):</t>
+        </is>
+      </c>
+      <c r="B6" s="46" t="n">
+        <v>945272.4347593583</v>
+      </c>
+      <c r="C6" s="38" t="inlineStr">
+        <is>
+          <t>&lt;- esse é o número que é de fato comparável a uma venda doméstica nos EUA (sem imposto de importação/consumo do Brasil).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Preço Final ao Cliente (com todos os impostos brasileiros):</t>
+        </is>
+      </c>
+      <c r="B7" s="46" t="n">
+        <v>1405909.269713061</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Diferença vs. referência EUA (Preço Líquido):</t>
+        </is>
+      </c>
+      <c r="B8" s="4">
+        <f>B6-B5</f>
+        <v/>
+      </c>
+      <c r="C8" s="47">
+        <f>B8/B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Diferença vs. referência EUA (Preço Final ao Cliente):</t>
+        </is>
+      </c>
+      <c r="B9" s="4">
+        <f>B7-B5</f>
+        <v/>
+      </c>
+      <c r="C9" s="47">
+        <f>B9/B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="38" t="inlineStr">
+        <is>
+          <t>PONTO-CHAVE: nosso Preço Líquido está próximo do preço de referência dos EUA - o salto grande até o Preço Final ao Cliente vem</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="38" t="inlineStr">
+        <is>
+          <t>inteiro do Imposto de Importação (II) e dos impostos de consumo brasileiros (IPI/PIS/COFINS/ICMS), que não existem numa venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="38" t="inlineStr">
+        <is>
+          <t>doméstica nos EUA e incidiriam do mesmo jeito seja importando componentes ou um vagão pronto (um veículo pronto pode inclusive</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="38" t="inlineStr">
+        <is>
+          <t>cair numa faixa de II diferente/maior - vale confirmar com um especialista em importação automotiva/ferroviária antes de assumir que 'comprar pronto' evita essa cascata de imposto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t>1) CASCATA COMPLETA (bate com a aba 'Resumo Executivo (P&amp;L)', só que com a fonte de cada linha)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="34" t="inlineStr">
+        <is>
+          <t>Etapa</t>
+        </is>
+      </c>
+      <c r="B16" s="34" t="inlineStr">
+        <is>
+          <t>Fórmula / Lógica</t>
+        </is>
+      </c>
+      <c r="C16" s="34" t="inlineStr">
+        <is>
+          <t>BRL</t>
+        </is>
+      </c>
+      <c r="D16" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E16" s="34" t="inlineStr">
+        <is>
+          <t>Multiplicador Acumulado</t>
+        </is>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>Fonte / Justificativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Raw Cost - Itens Importados</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>BOM USD unitário x Qtd x Câmbio, somado nos 47 itens importados precificados</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>1346980.92</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>264113.905882353</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.00x</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Aba Final Cost List, coluna F (BOM Price USD Unit) x coluna E (Quantity), câmbio da aba 'RATES' do Material Pricing.xlsm</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Raw Cost - Itens PAC</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Soma do custo unitário PAC (BRL) x Qtd nos 88 itens PAC</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>166060.16</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>32560.81568627451</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>9.11x</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Campo 'aco_cost' do 7-PAC Item Costs.xlsx por item, já é custo de fabricação local completo (material+mão de obra+overhead)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TP - Transfer Price</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>13% nos itens que já tinham algum TP historicamente; 17,2% nos que não tinham nenhum</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>198163.69</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>38855.62549019608</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>8.64x</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Diretriz do Matheus nesta sessão; a divisão 17,2%/0% original veio da cópia colorida de revisão (amarelo/verde)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Frete Internacional</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>1,2295642% sobre (Raw Cost + TP)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>18998.55</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>3725.205882352941</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>91.07x</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>'Planilha de Custos de Importação - Pathfinder - Set 26.xlsx' (cotação do despachante China Gate), Frete+Seguro / Valor do Produto</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>II - Imposto de Importação</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Blended 17.96% sobre (Raw Cost+TP+Frete): taxa real por NCM pros 6 itens com NCM confirmado, pior caso 18% flat pros outros 41</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>280915.82</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>55081.53333333334</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>7.16x</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Aba 'II' do Material Pricing.xlsm (consulta real por NCM) + nossa taxa flat antiga como fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Frete Nacional</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Cotação real fixa pra remessa inteira (Santos -&gt; Betim/Contagem, MG)</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>21753.1</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>4265.313725490196</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>93.45x</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Cotação China Gate, aba 'Despesas de Importação': Siscomex, despachante, armazenagem, transporte rodoviário, Marinha Mercante, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Supermetal - Integração/Montagem GDT</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Custo direto: reforma do vagão (teto, porta, escada, chicotes, skid de baterias, tubulação Fastbrake, ar condicionado, lastro)</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>707790.6</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>138782.4705882353</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>3.87x</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Aba 'GDT Integration and Assembly', soma da coluna Direct Cost BRL (18 itens)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>CUSTO FINAL (com TP):</t>
+        </is>
+      </c>
+      <c r="C24" s="42" t="n">
+        <v>2740662.84</v>
+      </c>
+      <c r="D24" s="43" t="n">
+        <v>537384.8705882353</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="40" t="inlineStr">
+        <is>
+          <t>2) MARGEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Base p/ margem</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Custo Final - TP (o TP fica fora da nossa base de margem - é margem da WBT USA, não nossa)</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Aba Approval Summary do Material Pricing.xlsm: TDM = (TP + GM_BRZ) / Preço Líquido. Algebricamente isso equivale a calcular a margem sobre (custo - TP) e devolver o TP depois, que é o que essa linha faz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Margem alvo (TDM)</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Editável - ver célula B4 da aba Resumo Executivo (P&amp;L)</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Alvo do Matheus pra esse exercício: 45%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="41" t="inlineStr">
+        <is>
+          <t>PREÇO LÍQUIDO ('NOSSO PREÇO'):</t>
+        </is>
+      </c>
+      <c r="C29" s="42" t="n">
+        <v>4820889.417272727</v>
+      </c>
+      <c r="D29" s="43" t="n">
+        <v>945272.4347593583</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1.759x</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="40" t="inlineStr">
+        <is>
+          <t>3) IMPOSTOS DE SAÍDA (o cliente paga; não afetam nossa margem)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>PIS/COFINS</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Preço Líquido / (1 - 10.06%) - por dentro, taxa blended real por NCM</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Aba 'II' do Material Pricing.xlsm (PIS+COFINS real por NCM) pros itens conhecidos, pior caso 9,25% pro resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ICMS</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Subtotal anterior / (1 - 18%) - por dentro, empilhado sobre PIS/COFINS</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>18% flat, bate com o exemplo real da Material Pricing. AINDA NÃO validado contra a alíquota de ICMS específica do estado de destino do cliente (as abas Tabela ICMS / Aliquotas Basicas têm a matriz real origem-destino se precisar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>IPI</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Subtotal anterior x IPI% blended - somado por fora, não é por dentro</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>Aba 'II' do Material Pricing.xlsm (IPI real por NCM) pros itens conhecidos, pior caso 9,75% pro resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="41" t="inlineStr">
+        <is>
+          <t>PREÇO FINAL AO CLIENTE:</t>
+        </is>
+      </c>
+      <c r="C35" s="42" t="n">
+        <v>7170137.27553661</v>
+      </c>
+      <c r="D35" s="43" t="n">
+        <v>1405909.269713061</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2.616x</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="40" t="inlineStr">
+        <is>
+          <t>4) REGISTRO DE PREMISSAS (questione um input específico aqui, não o número todo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="34" t="inlineStr">
+        <is>
+          <t>Premissa</t>
+        </is>
+      </c>
+      <c r="B38" s="34" t="inlineStr">
+        <is>
+          <t>Valor Usado</t>
+        </is>
+      </c>
+      <c r="C38" s="34" t="inlineStr">
+        <is>
+          <t>Confiança</t>
+        </is>
+      </c>
+      <c r="D38" s="34" t="inlineStr">
+        <is>
+          <t>Onde pode estar errado</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Câmbio</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>5,10 BRL/USD</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Foto fixa do Material Pricing.xlsm; vai variar com o câmbio real na data da fatura</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Divisão da taxa de TP</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>13% / 17,2%</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Baixa-Média</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Divisão arbitrária escolhida nesta sessão, não vem de um documento oficial de política de transfer pricing da Wabtec</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Frete Internacional</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1,23% do valor</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Cotação real do despachante, mas é só uma simulação pelo próprio aviso da cotação - confirmar com booking real</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Frete Nacional</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>R$21.753,10 fixo</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Cotação real específica pra Santos-&gt;Betim/Contagem; muda se origem/destino mudar</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>II (Imposto de Importação)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>17,96% blended (6 de 47 itens importados com NCM real)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>41 dos 47 itens importados ainda usam o pior caso 18% padrão - sem NCM confirmado pra eles ainda</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>PIS/COFINS</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>10,06% blended</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Mesma lacuna de cobertura de NCM que o II</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>IPI</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>9,69% blended</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Mesma lacuna de cobertura de NCM que o II</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ICMS</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>18% flat</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Baixa-Média</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Não consultado por par origem-destino UF; taxa real pode ser menor (interestadual) ou ter redução RBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Total Deal Margin (TDM)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>45%</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>N/A - decisão de negócio</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Essa é a maior alavanca isolada do preço final - ver tabela de sensibilidade abaixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Itens PAC</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Tratados como um bloco único all-in, sem decompor TP/frete/duty</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Custo PAC é genuinamente um custo de fabricação local brasileiro, não uma transação de importação</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Itens faltantes</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>27 itens excluídos (ainda sem custo)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Preço final vai aumentar quando esses tiverem cotação - ver aba 'Missing Items'</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Supermetal / rollup GDT</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Tratado como custo local, sem imposto de importação (correto, é mão de obra+material brasileiro)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Ainda não inclui ISS (imposto sobre serviço) na parte de mão de obra - desconsiderado por enquanto a pedido do Matheus</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="40" t="inlineStr">
+        <is>
+          <t>5) SENSIBILIDADE DA MARGEM (mesma base de custo, TDM diferentes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="48" t="inlineStr">
+        <is>
+          <t>TDM</t>
+        </is>
+      </c>
+      <c r="B53" s="48" t="inlineStr">
+        <is>
+          <t>Preço Líquido (Nosso Preço) USD</t>
+        </is>
+      </c>
+      <c r="C53" s="48" t="inlineStr">
+        <is>
+          <t>Preço Final ao Cliente USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="47" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B54" s="4" t="n">
+        <v>751040.2613445378</v>
+      </c>
+      <c r="C54" s="4" t="n">
+        <v>1117026.612143629</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="47" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="B56" s="4" t="n">
+        <v>805823.6948717949</v>
+      </c>
+      <c r="C56" s="4" t="n">
+        <v>1198506.336073469</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="47" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B58" s="4" t="n">
+        <v>869737.7006535948</v>
+      </c>
+      <c r="C58" s="4" t="n">
+        <v>1293566.013991615</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="49" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="B60" s="50" t="n">
+        <v>945272.4347593583</v>
+      </c>
+      <c r="C60" s="50" t="n">
+        <v>1405909.269713061</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B62" s="4" t="n">
+        <v>1035914.115686275</v>
+      </c>
+      <c r="C62" s="4" t="n">
+        <v>1540721.176578796</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="47" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="B64" s="4" t="n">
+        <v>1146698.392374728</v>
+      </c>
+      <c r="C64" s="4" t="n">
+        <v>1705491.28497025</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="44" t="inlineStr">
+        <is>
+          <t>Notas:</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="38" t="inlineStr">
+        <is>
+          <t>- Esta aba é complementar à 'Resumo Executivo (P&amp;L)' - mesmos números, mas cada linha se explica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="38" t="inlineStr">
+        <is>
+          <t>- QQP (impostos de serviço) e ISS na parte de mão de obra da Supermetal foram desconsiderados por enquanto, a pedido - o preço final pode aumentar quando isso for incluído.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="D41:F41"/>
+    <mergeCell ref="D48:F48"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="D43:F43"/>
+    <mergeCell ref="D39:F39"/>
+    <mergeCell ref="D42:F42"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A68:F68"/>
+    <mergeCell ref="A67:F67"/>
+    <mergeCell ref="D50:F50"/>
+    <mergeCell ref="D44:F44"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="D46:F46"/>
+    <mergeCell ref="D40:F40"/>
+    <mergeCell ref="D45:F45"/>
+    <mergeCell ref="D49:F49"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix misleading multiplier column in the Price Calc Detail tab
The per-line "cumulative multiplier" in the cost build-up section
(Raw Cost, PAC, TP, Freight, II, Domestic Freight, Supermetal) was
computed as running-total / this-line's-value, which is meaningless
since those lines are summed, not multiplied. Replaced with "-" for
those additive lines, and kept the real multiplier only where a
multiplicative step actually happens: Final Cost (1.000x baseline) ->
Net Price (margin effect) -> Final Client Price (tax cascade effect).
</commit_message>
<xml_diff>
--- a/Lista_Final_Pathfinder_SKID_Custos_English_Updated.xlsx
+++ b/Lista_Final_Pathfinder_SKID_Custos_English_Updated.xlsx
@@ -18151,7 +18151,7 @@
       </c>
       <c r="E16" s="34" t="inlineStr">
         <is>
-          <t>Multiplicador Acumulado</t>
+          <t>Multiplicador vs. Custo Final (só nos totais)</t>
         </is>
       </c>
       <c r="F16" s="34" t="inlineStr">
@@ -18179,7 +18179,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.00x</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -18207,7 +18207,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>9.11x</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -18235,7 +18235,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>8.64x</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -18263,7 +18263,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>91.07x</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -18291,7 +18291,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>7.16x</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -18319,7 +18319,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>93.45x</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -18347,7 +18347,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3.87x</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -18367,6 +18367,11 @@
       </c>
       <c r="D24" s="43" t="n">
         <v>537384.8705882353</v>
+      </c>
+      <c r="E24" s="41" t="inlineStr">
+        <is>
+          <t>1.000x (baseline)</t>
+        </is>
       </c>
     </row>
     <row r="26">

</xml_diff>